<commit_message>
docs: v1.2.0.0 릴리즈 노트 + 이슈 노트 (ENH-036~041)
- Release_note.md: v1.2.0.0 릴리즈 항목 추가
- Issue_list.xlsx: ENH-036~041 이슈 6건 추가 (총 120건)

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Issue_list.xlsx
+++ b/Issue_list.xlsx
@@ -574,7 +574,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L115"/>
+  <dimension ref="A1:L121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -7406,6 +7406,354 @@
         </is>
       </c>
       <c r="L115" s="19" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="19" t="inlineStr">
+        <is>
+          <t>ENH-036</t>
+        </is>
+      </c>
+      <c r="B116" s="19" t="inlineStr">
+        <is>
+          <t>Backend</t>
+        </is>
+      </c>
+      <c r="C116" s="20" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="D116" s="21" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="E116" s="19" t="inlineStr">
+        <is>
+          <t>엑셀 Export 시트 분리 옵션 (split_sheets)</t>
+        </is>
+      </c>
+      <c r="F116" s="19" t="inlineStr">
+        <is>
+          <t>1.1.0.1</t>
+        </is>
+      </c>
+      <c r="G116" s="19" t="inlineStr">
+        <is>
+          <t>1.2.0.0</t>
+        </is>
+      </c>
+      <c r="H116" s="19" t="n"/>
+      <c r="I116" s="19" t="inlineStr">
+        <is>
+          <t>Export 시 모든 TC가 단일 시트에 출력됨, sheet_name별 분리 필요</t>
+        </is>
+      </c>
+      <c r="J116" s="19" t="inlineStr">
+        <is>
+          <t>split_sheets=true 파라미터 추가, sheet_name 기준 엑셀 탭 분리 생성 + 시트명 특수문자 치환</t>
+        </is>
+      </c>
+      <c r="K116" s="19" t="inlineStr">
+        <is>
+          <t>TC Export</t>
+        </is>
+      </c>
+      <c r="L116" s="19" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="19" t="inlineStr">
+        <is>
+          <t>ENH-037</t>
+        </is>
+      </c>
+      <c r="B117" s="19" t="inlineStr">
+        <is>
+          <t>Backend</t>
+        </is>
+      </c>
+      <c r="C117" s="20" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="D117" s="21" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="E117" s="19" t="inlineStr">
+        <is>
+          <t>issue_link/assignee 미사용 컬럼 제거</t>
+        </is>
+      </c>
+      <c r="F117" s="19" t="inlineStr">
+        <is>
+          <t>1.1.0.1</t>
+        </is>
+      </c>
+      <c r="G117" s="19" t="inlineStr">
+        <is>
+          <t>1.2.0.0</t>
+        </is>
+      </c>
+      <c r="H117" s="19" t="n"/>
+      <c r="I117" s="19" t="inlineStr">
+        <is>
+          <t>TestCase 모델에 issue_link, assignee 컬럼이 있으나 실제 사용하지 않음</t>
+        </is>
+      </c>
+      <c r="J117" s="19" t="inlineStr">
+        <is>
+          <t>모델/스키마에서 컬럼 삭제, 임포트 매핑(Excel/CSV/MD/Jira) _skip 처리, 그리드 컬럼 제거</t>
+        </is>
+      </c>
+      <c r="K117" s="19" t="inlineStr">
+        <is>
+          <t>TC 모델/임포트/익스포트/그리드</t>
+        </is>
+      </c>
+      <c r="L117" s="19" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="19" t="inlineStr">
+        <is>
+          <t>ENH-038</t>
+        </is>
+      </c>
+      <c r="B118" s="19" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="C118" s="20" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="D118" s="21" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="E118" s="19" t="inlineStr">
+        <is>
+          <t>Excel Export 옵션 모달 UI</t>
+        </is>
+      </c>
+      <c r="F118" s="19" t="inlineStr">
+        <is>
+          <t>1.1.0.1</t>
+        </is>
+      </c>
+      <c r="G118" s="19" t="inlineStr">
+        <is>
+          <t>1.2.0.0</t>
+        </is>
+      </c>
+      <c r="H118" s="19" t="n"/>
+      <c r="I118" s="19" t="inlineStr">
+        <is>
+          <t>Export 버튼 클릭 시 바로 다운로드됨, 시트 분리 옵션 선택 불가</t>
+        </is>
+      </c>
+      <c r="J118" s="19" t="inlineStr">
+        <is>
+          <t>Export 버튼 → 모달 팝업 (통합/분리 라디오 선택 → 다운로드)</t>
+        </is>
+      </c>
+      <c r="K118" s="19" t="inlineStr">
+        <is>
+          <t>TC Export UI</t>
+        </is>
+      </c>
+      <c r="L118" s="19" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="19" t="inlineStr">
+        <is>
+          <t>ENH-039</t>
+        </is>
+      </c>
+      <c r="B119" s="19" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="C119" s="20" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="D119" s="21" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="E119" s="19" t="inlineStr">
+        <is>
+          <t>프로젝트 설정 — 이름/설명 편집 기능</t>
+        </is>
+      </c>
+      <c r="F119" s="19" t="inlineStr">
+        <is>
+          <t>1.1.0.1</t>
+        </is>
+      </c>
+      <c r="G119" s="19" t="inlineStr">
+        <is>
+          <t>1.2.0.0</t>
+        </is>
+      </c>
+      <c r="H119" s="19" t="n"/>
+      <c r="I119" s="19" t="inlineStr">
+        <is>
+          <t>프로젝트 생성 후 이름/설명 수정 불가</t>
+        </is>
+      </c>
+      <c r="J119" s="19" t="inlineStr">
+        <is>
+          <t>ProjectSettings에 이름/설명 input + 저장 버튼 추가 (admin 전용)</t>
+        </is>
+      </c>
+      <c r="K119" s="19" t="inlineStr">
+        <is>
+          <t>프로젝트 설정</t>
+        </is>
+      </c>
+      <c r="L119" s="19" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="19" t="inlineStr">
+        <is>
+          <t>ENH-040</t>
+        </is>
+      </c>
+      <c r="B120" s="19" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="C120" s="20" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="D120" s="21" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="E120" s="19" t="inlineStr">
+        <is>
+          <t>TestRunManager result 컬럼 select 위젯 전환</t>
+        </is>
+      </c>
+      <c r="F120" s="19" t="inlineStr">
+        <is>
+          <t>1.1.0.1</t>
+        </is>
+      </c>
+      <c r="G120" s="19" t="inlineStr">
+        <is>
+          <t>1.2.0.0</t>
+        </is>
+      </c>
+      <c r="H120" s="19" t="n"/>
+      <c r="I120" s="19" t="inlineStr">
+        <is>
+          <t>result 셀이 AG Grid 셀 에디터 방식 — 더블클릭 필요, 직관성 떨어짐</t>
+        </is>
+      </c>
+      <c r="J120" s="19" t="inlineStr">
+        <is>
+          <t>editable:false + 네이티브 &lt;select&gt; cellRenderer로 변경, Shift+클릭 채우기 로직 개선</t>
+        </is>
+      </c>
+      <c r="K120" s="19" t="inlineStr">
+        <is>
+          <t>TestRun 결과 입력</t>
+        </is>
+      </c>
+      <c r="L120" s="19" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="19" t="inlineStr">
+        <is>
+          <t>ENH-041</t>
+        </is>
+      </c>
+      <c r="B121" s="19" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="C121" s="20" t="inlineStr">
+        <is>
+          <t>Trivial</t>
+        </is>
+      </c>
+      <c r="D121" s="21" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="E121" s="19" t="inlineStr">
+        <is>
+          <t>test_steps/expected_result 컬럼 flex 레이아웃</t>
+        </is>
+      </c>
+      <c r="F121" s="19" t="inlineStr">
+        <is>
+          <t>1.1.0.1</t>
+        </is>
+      </c>
+      <c r="G121" s="19" t="inlineStr">
+        <is>
+          <t>1.2.0.0</t>
+        </is>
+      </c>
+      <c r="H121" s="19" t="n"/>
+      <c r="I121" s="19" t="inlineStr">
+        <is>
+          <t>고정 width로 화면 크기에 따라 빈 공간 발생</t>
+        </is>
+      </c>
+      <c r="J121" s="19" t="inlineStr">
+        <is>
+          <t>minWidth + flex:2 적용, 화면 크기에 맞게 자동 확장</t>
+        </is>
+      </c>
+      <c r="K121" s="19" t="inlineStr">
+        <is>
+          <t>TC 그리드/TestRun 그리드</t>
+        </is>
+      </c>
+      <c r="L121" s="19" t="inlineStr">
         <is>
           <t>완료</t>
         </is>

</xml_diff>

<commit_message>
chore(log): 조인 키가 빈 행 10건에 Linear 이슈를 만들고 키를 채운다 (SYM-13 ~ SYM-22)
현재 상태 문장이 완료 조건 칸에 들어가 있던 PERF/ENH 10행은 제자리로 옮겼다.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FigcsmP85LkasfoHXsHcwK
</commit_message>
<xml_diff>
--- a/Issue_list.xlsx
+++ b/Issue_list.xlsx
@@ -421,7 +421,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:U136"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
     <col width="11" customWidth="1" min="2" max="2"/>
@@ -7502,6 +7502,11 @@
           <t>2026-04-06</t>
         </is>
       </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>enhancement</t>
+        </is>
+      </c>
       <c r="D106" t="inlineStr">
         <is>
           <t>Minor</t>
@@ -7517,6 +7522,11 @@
           <t>대시보드 SQL 집계 전환 (ORM 전체 로드 → GROUP BY)</t>
         </is>
       </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>dashboard summary/priority/category/assignee/rounds/heatmap가 전체 ORM 객체를 Python에서 카운팅</t>
+        </is>
+      </c>
       <c r="K106" t="inlineStr">
         <is>
           <t>dashboard summary/priority/category/assignee/rounds/heatmap가 전체 ORM 객체를 Python에서 카운팅</t>
@@ -7545,6 +7555,11 @@
       <c r="T106" t="inlineStr">
         <is>
           <t>완료</t>
+        </is>
+      </c>
+      <c r="U106" t="inlineStr">
+        <is>
+          <t>SYM-13</t>
         </is>
       </c>
     </row>
@@ -7559,6 +7574,11 @@
           <t>2026-04-06</t>
         </is>
       </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>enhancement</t>
+        </is>
+      </c>
       <c r="D107" t="inlineStr">
         <is>
           <t>Minor</t>
@@ -7574,6 +7594,11 @@
           <t>Overview SQL 집계 전환 (Python 카운팅 → SQL 서브쿼리)</t>
         </is>
       </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>overview 엔드포인트가 전체 TestResult ORM 로드 후 Python _count_results로 집계</t>
+        </is>
+      </c>
       <c r="K107" t="inlineStr">
         <is>
           <t>overview 엔드포인트가 전체 TestResult ORM 로드 후 Python _count_results로 집계</t>
@@ -7602,6 +7627,11 @@
       <c r="T107" t="inlineStr">
         <is>
           <t>완료</t>
+        </is>
+      </c>
+      <c r="U107" t="inlineStr">
+        <is>
+          <t>SYM-14</t>
         </is>
       </c>
     </row>
@@ -7616,6 +7646,11 @@
           <t>2026-04-06</t>
         </is>
       </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>enhancement</t>
+        </is>
+      </c>
       <c r="D108" t="inlineStr">
         <is>
           <t>Minor</t>
@@ -7631,6 +7666,11 @@
           <t>TestPlan 목록 N+1 제거 (플랜별 개별 조회 → SQL 2회)</t>
         </is>
       </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>list_test_plans에서 플랜마다 run_count + _plan_progress 개별 DB 조회 (N+1)</t>
+        </is>
+      </c>
       <c r="K108" t="inlineStr">
         <is>
           <t>list_test_plans에서 플랜마다 run_count + _plan_progress 개별 DB 조회 (N+1)</t>
@@ -7659,6 +7699,11 @@
       <c r="T108" t="inlineStr">
         <is>
           <t>완료</t>
+        </is>
+      </c>
+      <c r="U108" t="inlineStr">
+        <is>
+          <t>SYM-15</t>
         </is>
       </c>
     </row>
@@ -7673,6 +7718,11 @@
           <t>2026-04-06</t>
         </is>
       </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>enhancement</t>
+        </is>
+      </c>
       <c r="D109" t="inlineStr">
         <is>
           <t>Minor</t>
@@ -7688,6 +7738,11 @@
           <t>TestRun 생성/복제 bulk insert 적용</t>
         </is>
       </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>create_testrun/clone에서 TC당 개별 db.add() — 5000건 시 ~7초</t>
+        </is>
+      </c>
       <c r="K109" t="inlineStr">
         <is>
           <t>create_testrun/clone에서 TC당 개별 db.add() — 5000건 시 ~7초</t>
@@ -7716,6 +7771,11 @@
       <c r="T109" t="inlineStr">
         <is>
           <t>완료</t>
+        </is>
+      </c>
+      <c r="U109" t="inlineStr">
+        <is>
+          <t>SYM-16</t>
         </is>
       </c>
     </row>
@@ -7730,6 +7790,11 @@
           <t>2026-04-06</t>
         </is>
       </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>enhancement</t>
+        </is>
+      </c>
       <c r="D110" t="inlineStr">
         <is>
           <t>Minor</t>
@@ -7745,6 +7810,11 @@
           <t>결과 제출 N+1 제거 (per-item .first() → IN prefetch)</t>
         </is>
       </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>submit_results에서 결과마다 기존 레코드를 개별 .first()로 조회</t>
+        </is>
+      </c>
       <c r="K110" t="inlineStr">
         <is>
           <t>submit_results에서 결과마다 기존 레코드를 개별 .first()로 조회</t>
@@ -7773,6 +7843,11 @@
       <c r="T110" t="inlineStr">
         <is>
           <t>완료</t>
+        </is>
+      </c>
+      <c r="U110" t="inlineStr">
+        <is>
+          <t>SYM-17</t>
         </is>
       </c>
     </row>
@@ -7787,6 +7862,11 @@
           <t>2026-04-06</t>
         </is>
       </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>enhancement</t>
+        </is>
+      </c>
       <c r="D111" t="inlineStr">
         <is>
           <t>Minor</t>
@@ -7802,6 +7882,11 @@
           <t>리포트 SQL 집계 + 이중 로드 제거</t>
         </is>
       </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>report Excel에서 _build_report_data + 별도 db.query 이중 로드, summary를 Python 카운팅</t>
+        </is>
+      </c>
       <c r="K111" t="inlineStr">
         <is>
           <t>report Excel에서 _build_report_data + 별도 db.query 이중 로드, summary를 Python 카운팅</t>
@@ -7830,6 +7915,11 @@
       <c r="T111" t="inlineStr">
         <is>
           <t>완료</t>
+        </is>
+      </c>
+      <c r="U111" t="inlineStr">
+        <is>
+          <t>SYM-18</t>
         </is>
       </c>
     </row>
@@ -7844,6 +7934,11 @@
           <t>2026-04-06</t>
         </is>
       </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>enhancement</t>
+        </is>
+      </c>
       <c r="D112" t="inlineStr">
         <is>
           <t>Trivial</t>
@@ -7859,6 +7954,11 @@
           <t>SQLite WAL 모드 활성화</t>
         </is>
       </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>SQLite 기본 journal_mode=delete, 동시 읽기/쓰기 시 lock</t>
+        </is>
+      </c>
       <c r="K112" t="inlineStr">
         <is>
           <t>SQLite 기본 journal_mode=delete, 동시 읽기/쓰기 시 lock</t>
@@ -7887,6 +7987,11 @@
       <c r="T112" t="inlineStr">
         <is>
           <t>완료</t>
+        </is>
+      </c>
+      <c r="U112" t="inlineStr">
+        <is>
+          <t>SYM-19</t>
         </is>
       </c>
     </row>
@@ -7901,6 +8006,11 @@
           <t>2026-04-06</t>
         </is>
       </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>enhancement</t>
+        </is>
+      </c>
       <c r="D113" t="inlineStr">
         <is>
           <t>Trivial</t>
@@ -7916,6 +8026,11 @@
           <t>시트 트리 순회 N+1 제거 (_collect_descendant_names)</t>
         </is>
       </c>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>_collect_descendant_names에서 재귀 while 루프로 시트마다 개별 DB 조회</t>
+        </is>
+      </c>
       <c r="K113" t="inlineStr">
         <is>
           <t>_collect_descendant_names에서 재귀 while 루프로 시트마다 개별 DB 조회</t>
@@ -7944,6 +8059,11 @@
       <c r="T113" t="inlineStr">
         <is>
           <t>완료</t>
+        </is>
+      </c>
+      <c r="U113" t="inlineStr">
+        <is>
+          <t>SYM-20</t>
         </is>
       </c>
     </row>
@@ -7958,6 +8078,11 @@
           <t>2026-04-06</t>
         </is>
       </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>enhancement</t>
+        </is>
+      </c>
       <c r="D114" t="inlineStr">
         <is>
           <t>Trivial</t>
@@ -7973,6 +8098,11 @@
           <t>ProjectPage 탭 lazy 분리 (초기 번들 ~120KB 절감)</t>
         </is>
       </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>ProjectPage에서 6개 탭 컴포넌트를 정적 import — 프로젝트 진입 시 전체 로드</t>
+        </is>
+      </c>
       <c r="K114" t="inlineStr">
         <is>
           <t>ProjectPage에서 6개 탭 컴포넌트를 정적 import — 프로젝트 진입 시 전체 로드</t>
@@ -8001,6 +8131,11 @@
       <c r="T114" t="inlineStr">
         <is>
           <t>완료</t>
+        </is>
+      </c>
+      <c r="U114" t="inlineStr">
+        <is>
+          <t>SYM-21</t>
         </is>
       </c>
     </row>
@@ -8015,6 +8150,11 @@
           <t>2026-04-06</t>
         </is>
       </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>enhancement</t>
+        </is>
+      </c>
       <c r="D115" t="inlineStr">
         <is>
           <t>Trivial</t>
@@ -8030,6 +8170,11 @@
           <t>번들 chunk 세분화 (index 638KB → 356KB)</t>
         </is>
       </c>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>vite manualChunks가 vendor/grid 2개만 분리, index 638KB</t>
+        </is>
+      </c>
       <c r="K115" t="inlineStr">
         <is>
           <t>vite manualChunks가 vendor/grid 2개만 분리, index 638KB</t>
@@ -8058,6 +8203,11 @@
       <c r="T115" t="inlineStr">
         <is>
           <t>완료</t>
+        </is>
+      </c>
+      <c r="U115" t="inlineStr">
+        <is>
+          <t>SYM-22</t>
         </is>
       </c>
     </row>
@@ -9699,6 +9849,7 @@
         <v>94</v>
       </c>
     </row>
+    <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
@@ -9756,6 +9907,7 @@
         <v>18</v>
       </c>
     </row>
+    <row r="15"/>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
docs: v1.3.2.0 릴리즈 노트와 이슈 11건 기록 (SYM-23 ~ SYM-33)
2026-09-07 에 올린 커밋 6건이 릴리즈 노트에도 트래커에도 없었다.
회사 PC 에서 작업해 기록 절차가 걸리지 않았다.

- Linear 이슈 11건 등록 후 닫음. 엑셀 로그 137~147행에 조인 키까지 채움
- 릴리즈 노트 v1.3.2.0 섹션 추가 (1,591자, A급 상한 1,600자 이내)
- 컴포넌트 버전: FE 1.3.0.0 -> 1.3.1.0, BE 1.3.1.0 -> 1.3.2.0,
  DB 0.7.1.0 -> 0.7.2.0, System 1.3.1.0 -> 1.3.2.0
- rules/versioning.md 이력 표에 빠져 있던 v1.3.0.1, v1.3.1.0 도 함께 채움
- package-lock 이 1.2.2.0 에 머물러 package.json 과 어긋나 있어 같이 맞춤

코드 변경 없음. 버전 문자열과 문서, 이슈 로그만 바뀐다.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CjcyQYfFMXsnLn4u9ktMkH
</commit_message>
<xml_diff>
--- a/Issue_list.xlsx
+++ b/Issue_list.xlsx
@@ -420,8 +420,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U136"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <dimension ref="A1:U147"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
     <col width="11" customWidth="1" min="2" max="2"/>
@@ -9768,6 +9768,1214 @@
         </is>
       </c>
     </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>BUG-078</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>bug</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>critical</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>db</t>
+        </is>
+      </c>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t>TC ID 가 프로젝트 안에서 중복돼 사전조건 참조가 엉뚱한 TC 를 가리킨다</t>
+        </is>
+      </c>
+      <c r="G137" t="inlineStr">
+        <is>
+          <t>- 한 프로젝트 안에 같은 TC ID 를 가진 TC 가 둘 이상 생긴다.
+- 사전조건 참조(`&lt;TC-ID&gt; 의 사전조건 참조`)를 푸는 색인이 프로젝트 전체 TC 로 만들어져서, 중복이 있으면 참조가 어느 쪽을 가리키는지 정해지지 않는다.</t>
+        </is>
+      </c>
+      <c r="H137" t="inlineStr">
+        <is>
+          <t>- TC ID 는 프로젝트 안에서 유일하다.
+- 사전조건 참조는 언제 풀어도 같은 TC 를 가리킨다.</t>
+        </is>
+      </c>
+      <c r="I137" t="inlineStr">
+        <is>
+          <t>- 내보내기의 펼친 사전조건이 참조 대상이 아닌 다른 TC 의 내용을 담는다. 데이터 손상이다.</t>
+        </is>
+      </c>
+      <c r="J137" t="inlineStr">
+        <is>
+          <t>- 프로젝트에 사전조건 참조를 쓰는 TC 가 있다.</t>
+        </is>
+      </c>
+      <c r="K137" t="inlineStr">
+        <is>
+          <t>1. 같은 TC ID 가 든 파일을 두 번 임포트한다.
+2. 또는 다른 시트에 같은 TC ID 로 임포트한다.
+3. 또는 TC 하나를 두 번 복제한다.
+4. 사전조건 참조를 쓰는 TC 를 엑셀로 내보낸다.
+5. 펼쳐진 사전조건 내용을 원본과 대조한다.</t>
+        </is>
+      </c>
+      <c r="L137" t="inlineStr">
+        <is>
+          <t>- 항상</t>
+        </is>
+      </c>
+      <c r="M137" t="inlineStr">
+        <is>
+          <t>- `precondition_service.build_index` 가 프로젝트 전체 TC 로 색인을 만든다.
+- `import_service` 의 `existing_map` 은 루프 시작 전 스냅샷이라 루프 안에서 새로 만든 행을 다시 담지 않는다.
+- 같은 `existing_map` 이 시트 단위인데 유일성 요구는 프로젝트 단위다.</t>
+        </is>
+      </c>
+      <c r="N137" t="inlineStr">
+        <is>
+          <t>- 코드 리뷰</t>
+        </is>
+      </c>
+      <c r="O137" t="inlineStr">
+        <is>
+          <t>원인: 중복이 생기는 경로가 넷이었고 넷 다 막혀 있지 않았다.
+- 임포트: `existing_map` 이 루프 시작 전 스냅샷이고 시트 단위였다.
+- 복제: `tc_id` 를 `{원본}-copy` 로 고정해 두 번 복제하면 겹쳤다.
+- 복원: 지운 사이에 같은 ID 가 새로 생겼으면 겹쳤다.
+- DB: `(project_id, tc_id)` 유니크 제약이 없었다.
+수정 내용: - 세 파서 모두 프로젝트 전체 `taken` 집합을 들고 다니며 빈 번호를 찾는다.
+- 복제가 원본 ID 에서 빈 번호를 새로 찾는다.
+- 복원이 `deleted_at` 을 풀기 전에 `taken` 을 조회한다(autoflush 때문에 순서가 중요하다).
+- 마이그레이션 `b7d3c9a1e450`: `(project_id, tc_id)` 부분 유니크 인덱스. `deleted_at IS NULL` 조건이 없으면 지운 TC 가 ID 를 계속 물어 같은 번호를 다시 못 쓴다.
+- 마이그레이션이 인덱스를 걸기 전에 중복을 스스로 정리한다. 가장 먼저 만든 행이 원래 ID 를 지키고 나머지에 `-2`, `-3` 을 붙이며 바꾼 내역을 WARNING 으로 남긴다. 앱 기동 시 자동 실행되므로(main.py lifespan) 여기서 실패하면 앱이 아예 뜨지 않는다.
+- 중복 시도가 500 이 아니라 409 와 안내 문구를 받게 IntegrityError 핸들러를 붙였다.
+- `services/tc_id_service.py` 신설.</t>
+        </is>
+      </c>
+      <c r="P137" t="inlineStr">
+        <is>
+          <t>- DB 부분 유니크 인덱스로 네 경로를 한 자리에서 막는다.
+- `backend/tests_unit/` 신설. `test_tc_id_dedup.py`, `test_unique_tc_id_migration.py`.
+- `backend/conftest.py` 의 `_server` 픽스처는 8008 에 서버가 떠 있으면 그 서버를 쓰고 admin 을 시드해서, 개발 서버를 켠 채로 pytest 를 돌리면 실 DB 에 쓰기가 들어간다. 같은 이름 픽스처를 no-op 으로 덮어 그 경로를 막았고 각 테스트는 임시 DB 만 쓴다.</t>
+        </is>
+      </c>
+      <c r="Q137" t="inlineStr">
+        <is>
+          <t>- TC 임포트, 복제, 복원, 사전조건 참조 해석, 엑셀 내보내기.
+- 기존 DB 에 중복이 있으면 첫 기동 때 ID 가 `-2`, `-3` 으로 바뀐다.</t>
+        </is>
+      </c>
+      <c r="R137" t="inlineStr">
+        <is>
+          <t>BE 1.3.1.0</t>
+        </is>
+      </c>
+      <c r="S137" t="inlineStr">
+        <is>
+          <t>- BE 1.3.2.0 / DB 0.7.2.0 (커밋: a92ca4c)</t>
+        </is>
+      </c>
+      <c r="T137" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="U137" t="inlineStr">
+        <is>
+          <t>SYM-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>BUG-079</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>bug</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>major</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>frontend</t>
+        </is>
+      </c>
+      <c r="F138" t="inlineStr">
+        <is>
+          <t>Expected Result 가 경고 없이 200자에서 잘린다</t>
+        </is>
+      </c>
+      <c r="G138" t="inlineStr">
+        <is>
+          <t>- 그리드에서 Expected Result 를 200자 넘게 입력하거나 붙여넣으면 200자까지만 들어간다.
+- 잘렸다는 경고가 없다.</t>
+        </is>
+      </c>
+      <c r="H138" t="inlineStr">
+        <is>
+          <t>- 길이 제한 없이 입력되고 그대로 저장된다. 백엔드 컬럼은 Text 라 제한이 없다.</t>
+        </is>
+      </c>
+      <c r="I138" t="inlineStr">
+        <is>
+          <t>- 201자째부터 사라진 채 저장된다.</t>
+        </is>
+      </c>
+      <c r="K138" t="inlineStr">
+        <is>
+          <t>1. TC 그리드에서 Expected Result 셀을 편집한다.
+2. 200자가 넘는 텍스트를 붙여넣는다.
+3. 셀을 빠져나온 뒤 값을 확인한다.</t>
+        </is>
+      </c>
+      <c r="L138" t="inlineStr">
+        <is>
+          <t>- 항상</t>
+        </is>
+      </c>
+      <c r="M138" t="inlineStr">
+        <is>
+          <t>- ag-grid `agLargeTextCellEditor` 는 `cellEditorParams.maxLength` 를 주지 않으면 textarea 에 `maxlength="200"` 을 박는다(`setMaxLength(maxLength || 200)`).</t>
+        </is>
+      </c>
+      <c r="N138" t="inlineStr">
+        <is>
+          <t>- 사용자</t>
+        </is>
+      </c>
+      <c r="O138" t="inlineStr">
+        <is>
+          <t>원인: - `agLargeTextCellEditor` 를 쓰면서 `cellEditorParams.maxLength` 를 주지 않았다. 라이브러리 기본값 200 이 그대로 걸렸다.
+수정 내용: - `utils/gridEditors.ts` 를 만들어 대용량 텍스트 편집기의 `maxLength` 를 명시한다. 백엔드 컬럼이 Text 이므로 편집기 쪽 제한만 푼다.</t>
+        </is>
+      </c>
+      <c r="P138" t="inlineStr">
+        <is>
+          <t>- 편집기 설정을 `utils/gridEditors.ts` 한 곳으로 모아 컬럼마다 빠뜨리지 않게 했다.</t>
+        </is>
+      </c>
+      <c r="Q138" t="inlineStr">
+        <is>
+          <t>- TC 그리드의 Expected Result 등 대용량 텍스트 컬럼 전체.
+- 이미 잘려 저장된 값은 복구되지 않는다.</t>
+        </is>
+      </c>
+      <c r="R138" t="inlineStr">
+        <is>
+          <t>FE 1.3.0.0</t>
+        </is>
+      </c>
+      <c r="S138" t="inlineStr">
+        <is>
+          <t>FE 1.3.1.0 (커밋: b66edeb)</t>
+        </is>
+      </c>
+      <c r="T138" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="U138" t="inlineStr">
+        <is>
+          <t>SYM-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>BUG-080</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>bug</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>major</t>
+        </is>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>frontend</t>
+        </is>
+      </c>
+      <c r="F139" t="inlineStr">
+        <is>
+          <t>Remarks 를 편집하면 줄바꿈이 사라진 채 저장된다</t>
+        </is>
+      </c>
+      <c r="G139" t="inlineStr">
+        <is>
+          <t>- 여러 줄로 쓴 비고를 그리드에서 편집하면 줄바꿈이 전부 사라진다.</t>
+        </is>
+      </c>
+      <c r="H139" t="inlineStr">
+        <is>
+          <t>- 여러 줄 비고가 줄바꿈을 유지한 채 저장되고, 렌더러가 줄 단위로 보여 준다.</t>
+        </is>
+      </c>
+      <c r="I139" t="inlineStr">
+        <is>
+          <t>- 한 줄로 이어붙은 채 저장된다.</t>
+        </is>
+      </c>
+      <c r="K139" t="inlineStr">
+        <is>
+          <t>1. Remarks 셀에 두 줄 이상을 넣는다.
+2. 저장 후 다시 편집한다.
+3. 저장된 값에서 줄바꿈이 사라진 것을 확인한다.</t>
+        </is>
+      </c>
+      <c r="L139" t="inlineStr">
+        <is>
+          <t>- 항상</t>
+        </is>
+      </c>
+      <c r="M139" t="inlineStr">
+        <is>
+          <t>- Remarks 컬럼에 `cellEditor` 가 없어 기본 편집기 `&lt;input type="text"&gt;` 가 붙었다. HTML 명세상 text input 은 값에서 줄바꿈을 제거한다.
+- 운영 DB 에 줄바꿈이 든 `remarks` 가 0건이었다.
+- 렌더러 `MarkdownCell` 이 값을 `split("\n")` 하는 것을 보면 여러 줄이 전제였다.</t>
+        </is>
+      </c>
+      <c r="N139" t="inlineStr">
+        <is>
+          <t>- 코드 리뷰</t>
+        </is>
+      </c>
+      <c r="O139" t="inlineStr">
+        <is>
+          <t>원인: - Remarks 컬럼에 `cellEditor` 지정이 빠져 단일행 text input 이 붙었다.
+수정 내용: - Remarks 에 대용량 텍스트 편집기를 붙이고 `maxLength` 를 함께 명시한다.</t>
+        </is>
+      </c>
+      <c r="P139" t="inlineStr">
+        <is>
+          <t>- 여러 줄을 전제로 렌더링하는 컬럼은 `utils/gridEditors.ts` 의 같은 편집기를 쓰게 통일했다.</t>
+        </is>
+      </c>
+      <c r="Q139" t="inlineStr">
+        <is>
+          <t>- TC 그리드 Remarks 컬럼.
+- 이미 한 줄로 눌린 기존 값은 복구되지 않는다.</t>
+        </is>
+      </c>
+      <c r="R139" t="inlineStr">
+        <is>
+          <t>FE 1.3.0.0</t>
+        </is>
+      </c>
+      <c r="S139" t="inlineStr">
+        <is>
+          <t>FE 1.3.1.0 (커밋: b66edeb)</t>
+        </is>
+      </c>
+      <c r="T139" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="U139" t="inlineStr">
+        <is>
+          <t>SYM-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>BUG-081</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>bug</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>major</t>
+        </is>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>frontend</t>
+        </is>
+      </c>
+      <c r="F140" t="inlineStr">
+        <is>
+          <t>TC ID 자동채우기가 한 행도 채우지 않는데 완료 토스트가 뜬다</t>
+        </is>
+      </c>
+      <c r="G140" t="inlineStr">
+        <is>
+          <t>- 여러 행을 선택해 TC ID 자동채우기를 실행하면 아무 행도 채워지지 않는다.
+- 그런데도 완료 토스트가 뜬다.</t>
+        </is>
+      </c>
+      <c r="H140" t="inlineStr">
+        <is>
+          <t>- 선택한 첫 행을 기준점으로 잡고 나머지 행에 이어지는 번호가 들어간다.
+- 채운 행이 없으면 없다고 알린다.</t>
+        </is>
+      </c>
+      <c r="I140" t="inlineStr">
+        <is>
+          <t>- 채워진 행이 0개인데 성공으로 보고된다.</t>
+        </is>
+      </c>
+      <c r="K140" t="inlineStr">
+        <is>
+          <t>1. TC 그리드에서 TC ID 가 빈 행을 여러 개 선택한다.
+2. TC ID 자동채우기를 실행한다.
+3. 완료 토스트가 뜨지만 TC ID 칸이 그대로인 것을 확인한다.</t>
+        </is>
+      </c>
+      <c r="L140" t="inlineStr">
+        <is>
+          <t>- 항상</t>
+        </is>
+      </c>
+      <c r="M140" t="inlineStr">
+        <is>
+          <t>- 선택 행마다 기준점을 다시 잡고 `continue` 해서 실제 대입에 도달하지 않았다.
+- 중복 판단이 화면 행 기준이었다. `getSelectedRows()` 는 필터로 숨은 선택 행까지 돌려주는데(selectedNodes 를 그대로 뱉는다) `allRows` 는 `forEachNodeAfterFilterAndSort` 로 만들어져서, 숨은 행과 ID 가 겹쳐도 경고가 뜨지 않았다.</t>
+        </is>
+      </c>
+      <c r="N140" t="inlineStr">
+        <is>
+          <t>- 사용자</t>
+        </is>
+      </c>
+      <c r="O140" t="inlineStr">
+        <is>
+          <t>원인: - 순번 계산이 그리드 컴포넌트에 인라인으로 박혀 있었고 테스트가 없었다. 기준점을 행마다 다시 잡는 분기가 남아 있어 아무것도 채우지 못했다.
+수정 내용: - 기준점은 선택 첫 행 하나만 쓰고 나머지를 이어 채운다.
+- 판단 근거를 화면 행에서 전체 행으로 옮기고, 숨어서 건너뛴 선택 행 수를 알려 준다.
+- 되돌릴 수 있게 undo 스택에 넣는다(기존에는 `pushUndo` 호출이 아예 없었다).
+- 행 식별 키를 `(id || no)` 에서 접두사를 붙인 형태로 바꿔 id 와 no 가 같은 숫자일 때의 충돌을 없앴다.
+- 순번 계산을 `utils/tcId.ts` 로 떼어냈다.</t>
+        </is>
+      </c>
+      <c r="P140" t="inlineStr">
+        <is>
+          <t>- `frontend/src/test/tcId.test.ts` 21건. 그리드에 인라인으로 박혀 테스트가 없던 것이 이 결함이 남아 있던 이유다.</t>
+        </is>
+      </c>
+      <c r="Q140" t="inlineStr">
+        <is>
+          <t>- TC 그리드의 TC ID 자동채우기, undo 스택.</t>
+        </is>
+      </c>
+      <c r="R140" t="inlineStr">
+        <is>
+          <t>FE 1.3.0.0</t>
+        </is>
+      </c>
+      <c r="S140" t="inlineStr">
+        <is>
+          <t>FE 1.3.1.0 (커밋: b66edeb)</t>
+        </is>
+      </c>
+      <c r="T140" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="U140" t="inlineStr">
+        <is>
+          <t>SYM-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>BUG-082</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>bug</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>major</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>frontend</t>
+        </is>
+      </c>
+      <c r="F141" t="inlineStr">
+        <is>
+          <t>행을 여러 개 추가하면 전부 같은 순번과 TC ID 를 받는다</t>
+        </is>
+      </c>
+      <c r="G141" t="inlineStr">
+        <is>
+          <t>- 대량 추가로 30행을 넣으면 30행이 전부 같은 `no` 와 같은 TC ID 를 갖는다.</t>
+        </is>
+      </c>
+      <c r="H141" t="inlineStr">
+        <is>
+          <t>- 추가한 행마다 순번과 TC ID 가 1씩 이어진다.</t>
+        </is>
+      </c>
+      <c r="I141" t="inlineStr">
+        <is>
+          <t>- 모든 행이 같은 값을 받아, 저장하면 TC ID 중복이 된다.</t>
+        </is>
+      </c>
+      <c r="K141" t="inlineStr">
+        <is>
+          <t>1. TC 그리드에서 행 대량 추가를 연다.
+2. 30행을 추가한다.
+3. 추가된 행들의 순번과 TC ID 를 확인한다.</t>
+        </is>
+      </c>
+      <c r="L141" t="inlineStr">
+        <is>
+          <t>- 항상</t>
+        </is>
+      </c>
+      <c r="M141" t="inlineStr">
+        <is>
+          <t>- 대량 추가가 `await` 루프로 `handleAddRow` 를 부르는데, 렌더 시점 `rowData` 를 클로저로 잡아 `nextNo` 가 루프 내내 같았다.
+- 접두사도 기존 행에서 가져오지 않고 `"TC-"` 로 고정돼 있었다.</t>
+        </is>
+      </c>
+      <c r="N141" t="inlineStr">
+        <is>
+          <t>- 사용자</t>
+        </is>
+      </c>
+      <c r="O141" t="inlineStr">
+        <is>
+          <t>원인: - 한 행 추가 함수를 루프로 부르면서 다음 순번을 클로저에 잡힌 옛 `rowData` 에서 계산했다.
+수정 내용: - `addRows(count)` 로 합쳐 다음 순번을 루프 밖에서 한 번만 계산한다.
+- 접두사를 기존 행에서 가져온다.</t>
+        </is>
+      </c>
+      <c r="P141" t="inlineStr">
+        <is>
+          <t>- 순번 계산이 `utils/tcId.ts` 로 빠지면서 같은 테스트 21건이 이 경로도 덮는다.</t>
+        </is>
+      </c>
+      <c r="Q141" t="inlineStr">
+        <is>
+          <t>- TC 그리드 행 추가와 대량 추가.
+- 이 경로로 만들어져 이미 저장된 중복 TC ID 는 마이그레이션 `b7d3c9a1e450` 이 `-2`, `-3` 으로 정리한다.</t>
+        </is>
+      </c>
+      <c r="R141" t="inlineStr">
+        <is>
+          <t>FE 1.3.0.0</t>
+        </is>
+      </c>
+      <c r="S141" t="inlineStr">
+        <is>
+          <t>FE 1.3.1.0 (커밋: b66edeb)</t>
+        </is>
+      </c>
+      <c r="T141" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="U141" t="inlineStr">
+        <is>
+          <t>SYM-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>BUG-083</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>bug</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>minor</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>frontend</t>
+        </is>
+      </c>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t>시트가 하나인 프로젝트에서 행을 추가하면 `기본` 시트가 조용히 생긴다</t>
+        </is>
+      </c>
+      <c r="G142" t="inlineStr">
+        <is>
+          <t>- 시트가 하나뿐인 프로젝트를 열고 바로 행을 추가하면, 만든 적 없는 `기본` 시트가 생기고 행이 그쪽으로 들어간다.</t>
+        </is>
+      </c>
+      <c r="H142" t="inlineStr">
+        <is>
+          <t>- 시트가 하나면 그 시트가 선택된 상태여야 하고, 행은 그 시트에 들어간다.</t>
+        </is>
+      </c>
+      <c r="I142" t="inlineStr">
+        <is>
+          <t>- `기본` 시트가 새로 만들어지고 행이 원래 시트에 보이지 않는다.</t>
+        </is>
+      </c>
+      <c r="J142" t="inlineStr">
+        <is>
+          <t>- 프로젝트에 시트가 하나만 있다.</t>
+        </is>
+      </c>
+      <c r="K142" t="inlineStr">
+        <is>
+          <t>1. 시트가 하나인 프로젝트를 연다.
+2. 시트를 직접 클릭하지 않고 바로 행을 추가한다.
+3. 시트 목록에 `기본` 이 생긴 것을 확인한다.</t>
+        </is>
+      </c>
+      <c r="L142" t="inlineStr">
+        <is>
+          <t>- 항상</t>
+        </is>
+      </c>
+      <c r="M142" t="inlineStr">
+        <is>
+          <t>- 시트 자동 선택 조건이 `flatAll.length &gt; 1` 이라 시트가 하나면 로드 직후 `activeSheet` 가 null 이었다.
+- 그 상태의 행 추가가 `sheet_name` 을 `기본` 으로 보내고 백엔드가 그 시트를 만들었다(`sheets.py` `auto_create_default`).</t>
+        </is>
+      </c>
+      <c r="N142" t="inlineStr">
+        <is>
+          <t>- 코드 리뷰</t>
+        </is>
+      </c>
+      <c r="O142" t="inlineStr">
+        <is>
+          <t>원인: - 시트 자동 선택 조건이 하나짜리 프로젝트를 빠뜨렸다.
+수정 내용: - 자동 선택 조건을 고쳐 시트가 하나여도 선택되게 했다.
+- `전체` 보기에서는 행 추가 버튼을 막는다.</t>
+        </is>
+      </c>
+      <c r="P142" t="inlineStr">
+        <is>
+          <t>- `전체` 보기에서 추가를 막아 시트가 정해지지 않은 상태로는 행을 만들 수 없게 했다.</t>
+        </is>
+      </c>
+      <c r="Q142" t="inlineStr">
+        <is>
+          <t>- 시트가 하나인 프로젝트의 행 추가.</t>
+        </is>
+      </c>
+      <c r="R142" t="inlineStr">
+        <is>
+          <t>FE 1.3.0.0</t>
+        </is>
+      </c>
+      <c r="S142" t="inlineStr">
+        <is>
+          <t>FE 1.3.1.0 (커밋: b66edeb)</t>
+        </is>
+      </c>
+      <c r="T142" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="U142" t="inlineStr">
+        <is>
+          <t>SYM-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>BUG-084</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>bug</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>minor</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>frontend</t>
+        </is>
+      </c>
+      <c r="F143" t="inlineStr">
+        <is>
+          <t>자동 저장이 실패해도 이유를 알려주지 않는다</t>
+        </is>
+      </c>
+      <c r="G143" t="inlineStr">
+        <is>
+          <t>- 그리드 자동 저장이 실패하면 `자동 저장 실패` 만 뜬다. 서버가 준 사유가 화면에 나오지 않는다.</t>
+        </is>
+      </c>
+      <c r="H143" t="inlineStr">
+        <is>
+          <t>- 서버가 준 `detail` 을 사용자 언어로 보여 준다. TC ID 중복이면 어느 ID 가 겹쳤는지 알 수 있어야 한다.</t>
+        </is>
+      </c>
+      <c r="I143" t="inlineStr">
+        <is>
+          <t>- 무엇을 고쳐야 하는지 알 수 없어 같은 편집을 반복하게 된다.</t>
+        </is>
+      </c>
+      <c r="K143" t="inlineStr">
+        <is>
+          <t>1. 이미 쓰이는 TC ID 를 다른 행에 입력한다.
+2. 자동 저장이 도는 것을 기다린다.
+3. 토스트 문구를 확인한다.</t>
+        </is>
+      </c>
+      <c r="L143" t="inlineStr">
+        <is>
+          <t>- 항상</t>
+        </is>
+      </c>
+      <c r="M143" t="inlineStr">
+        <is>
+          <t>- 자동 저장 실패 경로가 서버 응답의 `detail` 을 읽지 않고 고정 문구만 띄웠다.</t>
+        </is>
+      </c>
+      <c r="N143" t="inlineStr">
+        <is>
+          <t>- 코드 리뷰</t>
+        </is>
+      </c>
+      <c r="O143" t="inlineStr">
+        <is>
+          <t>원인: - 오류 처리에서 응답 본문을 버리고 고정 문구를 썼다.
+수정 내용: - 서버가 준 `detail` 을 `translateError` 로 옮겨 띄운다.
+- `utils/errorMessage.ts` 에 TC ID 중복 409 문구를 추가하고 ko/en 사전에 넣었다.</t>
+        </is>
+      </c>
+      <c r="P143" t="inlineStr">
+        <is>
+          <t>- 백엔드가 이 경우 500 이 아니라 409 와 안내 문구를 돌려주도록 함께 고쳤다(a92ca4c).</t>
+        </is>
+      </c>
+      <c r="Q143" t="inlineStr">
+        <is>
+          <t>- TC 그리드 자동 저장 오류 표시, ko/en 번역 사전.</t>
+        </is>
+      </c>
+      <c r="R143" t="inlineStr">
+        <is>
+          <t>FE 1.3.0.0</t>
+        </is>
+      </c>
+      <c r="S143" t="inlineStr">
+        <is>
+          <t>FE 1.3.1.0 (커밋: b66edeb)</t>
+        </is>
+      </c>
+      <c r="T143" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="U143" t="inlineStr">
+        <is>
+          <t>SYM-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>BUG-085</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>bug</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>minor</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>frontend</t>
+        </is>
+      </c>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>그리드 헤더의 필터 버튼이 배경과 대비가 없어 보이지 않는다</t>
+        </is>
+      </c>
+      <c r="G144" t="inlineStr">
+        <is>
+          <t>- 그리드 헤더의 필터 버튼이 사실상 검정 위 검정이라 어디를 눌러야 필터가 열리는지 보이지 않는다.</t>
+        </is>
+      </c>
+      <c r="H144" t="inlineStr">
+        <is>
+          <t>- 라이트와 다크 양쪽에서 헤더 글자와 같은 수준으로 읽힌다.</t>
+        </is>
+      </c>
+      <c r="I144" t="inlineStr">
+        <is>
+          <t>- 대비 약 1.1:1. 버튼이 있는지조차 알 수 없다.</t>
+        </is>
+      </c>
+      <c r="K144" t="inlineStr">
+        <is>
+          <t>1. TC 그리드를 연다.
+2. 헤더 셀에 마우스를 올린다.
+3. 필터 버튼을 찾아본다.</t>
+        </is>
+      </c>
+      <c r="L144" t="inlineStr">
+        <is>
+          <t>- 항상</t>
+        </is>
+      </c>
+      <c r="M144" t="inlineStr">
+        <is>
+          <t>- `.ag-header-cell-filter-button` 이 `--ag-foreground-color` 를 따라가 `#1A1D23` 으로 칠해졌다. 헤더 배경은 `#1E293B` 라 대비 약 1.1:1.
+- 같은 헤더의 필터 걸림 표시(`.ag-icon-filter`)는 헤더 전경색을 제대로 받고 있어서 버튼만 빠져 있었다.</t>
+        </is>
+      </c>
+      <c r="N144" t="inlineStr">
+        <is>
+          <t>- 사용자</t>
+        </is>
+      </c>
+      <c r="O144" t="inlineStr">
+        <is>
+          <t>원인: - 필터 버튼이 헤더 전경색이 아니라 본문 전경색 변수를 따라갔다.
+수정 내용: - `--ag-header-foreground-color` 를 따라가게 해서 라이트와 다크 양쪽에서 자동으로 맞는다(실측 13.35:1 / 15.01:1).
+- 아이콘이 `mask-image` + `background-color` 로 그려지므로 `::before` 도 같이 지정한다.
+- 평소 `opacity` 0.7, 셀 호버 시 1 로 올려 헤더 글자를 가리지 않게 했다.
+- 필터가 걸린 열은 파란색으로 칠해 어느 열에 필터가 있는지 바로 보이게 했다.</t>
+        </is>
+      </c>
+      <c r="P144" t="inlineStr">
+        <is>
+          <t>- 색을 고정값이 아니라 헤더 전경색 변수에 묶어 테마를 바꿔도 따라온다.</t>
+        </is>
+      </c>
+      <c r="Q144" t="inlineStr">
+        <is>
+          <t>- 그리드 헤더 필터 버튼 전체(라이트, 다크).</t>
+        </is>
+      </c>
+      <c r="R144" t="inlineStr">
+        <is>
+          <t>FE 1.3.0.0</t>
+        </is>
+      </c>
+      <c r="S144" t="inlineStr">
+        <is>
+          <t>FE 1.3.1.0 (커밋: b554e86)</t>
+        </is>
+      </c>
+      <c r="T144" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="U144" t="inlineStr">
+        <is>
+          <t>SYM-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>BUG-086</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>bug</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>blocker</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>db</t>
+        </is>
+      </c>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>alembic head 가 둘로 갈라져 앱이 기동하지 못한다</t>
+        </is>
+      </c>
+      <c r="G145" t="inlineStr">
+        <is>
+          <t>- 백엔드가 기동하지 못한다. `Multiple head revisions are present` 로 마이그레이션이 실패한다.</t>
+        </is>
+      </c>
+      <c r="H145" t="inlineStr">
+        <is>
+          <t>- `alembic upgrade head` 가 단일 head 로 통과하고 앱이 뜬다.</t>
+        </is>
+      </c>
+      <c r="I145" t="inlineStr">
+        <is>
+          <t>- 마이그레이션이 lifespan 안에서 터져 앱이 아예 뜨지 않는다. 우회 경로가 없다.</t>
+        </is>
+      </c>
+      <c r="K145" t="inlineStr">
+        <is>
+          <t>1. `b7d3c9a1e450` 이 포함된 커밋을 받는다.
+2. 백엔드를 기동한다.
+3. `Multiple head revisions are present` 를 확인한다.</t>
+        </is>
+      </c>
+      <c r="L145" t="inlineStr">
+        <is>
+          <t>- 항상</t>
+        </is>
+      </c>
+      <c r="M145" t="inlineStr">
+        <is>
+          <t>- 원격에 `05f8800a57f5`(account_requests)와 `a1c4e7b9d2f0`(test_results 유니크)이 먼저 올라가 있었다.
+- `b7d3c9a1e450` 의 `down_revision` 이 `06933fddb519` 이라 둘 다 같은 부모에서 갈라져 head 가 두 개가 됐다.</t>
+        </is>
+      </c>
+      <c r="N145" t="inlineStr">
+        <is>
+          <t>- 코드 리뷰</t>
+        </is>
+      </c>
+      <c r="O145" t="inlineStr">
+        <is>
+          <t>원인: - 마이그레이션을 로컬에서 만들 때 부모를 원격 최신 head 가 아니라 그 앞 리비전으로 잡았다.
+수정 내용: - `down_revision` 을 `a1c4e7b9d2f0` 으로 바꿔 체인 맨 뒤에 붙인다.</t>
+        </is>
+      </c>
+      <c r="P145" t="inlineStr">
+        <is>
+          <t>- 체인이 `8925bb1ad2db` -&gt; `06933fddb519` -&gt; `05f8800a57f5` -&gt; `a1c4e7b9d2f0` -&gt; `b7d3c9a1e450` 단일 선형인 것을 확인했다.
+- 마이그레이션이 lifespan 에서 자동 실행되므로 여기서 실패하면 앱 전체가 못 뜬다. 새 마이그레이션은 `alembic heads` 가 하나인지 보고 만든다.</t>
+        </is>
+      </c>
+      <c r="Q145" t="inlineStr">
+        <is>
+          <t>- 백엔드 기동 전체.</t>
+        </is>
+      </c>
+      <c r="R145" t="inlineStr">
+        <is>
+          <t>DB 0.7.2.0</t>
+        </is>
+      </c>
+      <c r="S145" t="inlineStr">
+        <is>
+          <t>DB 0.7.2.0 (커밋: a1f525e)</t>
+        </is>
+      </c>
+      <c r="T145" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="U145" t="inlineStr">
+        <is>
+          <t>SYM-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>SEC-014</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>bug</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>minor</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>security</t>
+        </is>
+      </c>
+      <c r="F146" t="inlineStr">
+        <is>
+          <t>로컬 자격증명 파일과 QA 스크래치 스크립트가 gitignore 에 없다</t>
+        </is>
+      </c>
+      <c r="G146" t="inlineStr">
+        <is>
+          <t>- `ym-testcase-credentials.txt` 와 `frontend/_*.mjs` 가 untracked 인데 무시 대상이 아니었다.</t>
+        </is>
+      </c>
+      <c r="H146" t="inlineStr">
+        <is>
+          <t>- 평문 계정 정보가 든 로컬 파일은 `git add -A` 로도 올라가지 않는다.</t>
+        </is>
+      </c>
+      <c r="I146" t="inlineStr">
+        <is>
+          <t>- `git add -A` 한 번에 공개 저장소로 올라갈 수 있는 상태였다.</t>
+        </is>
+      </c>
+      <c r="K146" t="inlineStr">
+        <is>
+          <t>1. 저장소 루트에서 `git status --porcelain` 을 본다.
+2. `ym-testcase-credentials.txt` 와 `frontend/_*.mjs` 가 `??` 로 잡히는 것을 확인한다.</t>
+        </is>
+      </c>
+      <c r="L146" t="inlineStr">
+        <is>
+          <t>- 항상</t>
+        </is>
+      </c>
+      <c r="M146" t="inlineStr">
+        <is>
+          <t>- 스크래치 스크립트 17개 중 14개에 평문 비밀번호와 계정 문자열이 들어 있었다.
+- 원격은 공개 저장소다.
+- 히스토리에 커밋된 적은 없음을 확인했다. 실제 유출은 없었다.</t>
+        </is>
+      </c>
+      <c r="N146" t="inlineStr">
+        <is>
+          <t>- 코드 리뷰</t>
+        </is>
+      </c>
+      <c r="O146" t="inlineStr">
+        <is>
+          <t>원인: - QA 작업 중 만든 로컬 파일들이 `.gitignore` 에 반영되지 않았다.
+수정 내용: - `.gitignore` 에 `ym-testcase-credentials.txt` 와 `frontend/_*.mjs` 를 포함한 5줄을 추가한다.</t>
+        </is>
+      </c>
+      <c r="P146" t="inlineStr">
+        <is>
+          <t>- 스크래치 파일 이름 규칙(`_` 접두사)을 통째로 무시 대상에 넣어 다음 파일도 자동으로 걸린다.</t>
+        </is>
+      </c>
+      <c r="Q146" t="inlineStr">
+        <is>
+          <t>- 저장소 전체. 이미 푸시된 내용은 없다.</t>
+        </is>
+      </c>
+      <c r="R146" t="inlineStr">
+        <is>
+          <t>System 1.3.1.0</t>
+        </is>
+      </c>
+      <c r="S146" t="inlineStr">
+        <is>
+          <t>System 1.3.2.0 (커밋: 160e924)</t>
+        </is>
+      </c>
+      <c r="T146" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="U146" t="inlineStr">
+        <is>
+          <t>SYM-32</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>BUG-087</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>bug</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>trivial</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>etc</t>
+        </is>
+      </c>
+      <c r="F147" t="inlineStr">
+        <is>
+          <t>package-lock 버전이 package.json 과 어긋난다</t>
+        </is>
+      </c>
+      <c r="G147" t="inlineStr">
+        <is>
+          <t>- `frontend/package-lock.json` 의 `version` 이 `package.json` 과 다르다. npm 을 실행할 때마다 lock 이 조용히 다시 쓰인다.</t>
+        </is>
+      </c>
+      <c r="H147" t="inlineStr">
+        <is>
+          <t>- 두 파일의 `version` 이 같아 npm 실행이 lock 을 건드리지 않는다.</t>
+        </is>
+      </c>
+      <c r="I147" t="inlineStr">
+        <is>
+          <t>- lock 이 `1.0.3.0` 에 머물러 있다가 npm 실행 시 `1.2.2.0` 으로 바뀌었고, `package.json` 은 `1.3.1.0` 이라 여전히 어긋났다.</t>
+        </is>
+      </c>
+      <c r="K147" t="inlineStr">
+        <is>
+          <t>1. `frontend/package.json` 과 `frontend/package-lock.json` 의 `version` 을 비교한다.
+2. `npm install` 을 돌린 뒤 `git status` 로 lock 이 변경되는지 본다.</t>
+        </is>
+      </c>
+      <c r="L147" t="inlineStr">
+        <is>
+          <t>- 항상</t>
+        </is>
+      </c>
+      <c r="M147" t="inlineStr">
+        <is>
+          <t>- 커밋 `fdc6e5f` 시점 diff: lock `1.0.3.0` -&gt; `1.2.2.0`, 같은 시점 `package.json` 은 `1.3.1.0`.</t>
+        </is>
+      </c>
+      <c r="N147" t="inlineStr">
+        <is>
+          <t>- 코드 리뷰</t>
+        </is>
+      </c>
+      <c r="O147" t="inlineStr">
+        <is>
+          <t>원인: - 릴리즈마다 `package.json` 만 올리고 lock 을 같이 올리지 않았다. 의존성 변경은 없다.
+수정 내용: - lock 의 두 `version` 필드를 `package.json` 과 같은 값으로 맞춘다.</t>
+        </is>
+      </c>
+      <c r="P147" t="inlineStr">
+        <is>
+          <t>- 버전 올릴 때 `package.json` 과 lock 의 두 자리를 함께 고친다.</t>
+        </is>
+      </c>
+      <c r="Q147" t="inlineStr">
+        <is>
+          <t>- 프론트엔드 빌드 메타데이터. 의존성 트리는 그대로다.</t>
+        </is>
+      </c>
+      <c r="R147" t="inlineStr">
+        <is>
+          <t>FE 1.3.0.0</t>
+        </is>
+      </c>
+      <c r="S147" t="inlineStr">
+        <is>
+          <t>FE 1.3.1.0 (커밋: fdc6e5f)</t>
+        </is>
+      </c>
+      <c r="T147" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="U147" t="inlineStr">
+        <is>
+          <t>SYM-33</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -9849,7 +11057,6 @@
         <v>94</v>
       </c>
     </row>
-    <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
@@ -9907,7 +11114,6 @@
         <v>18</v>
       </c>
     </row>
-    <row r="15"/>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
feat(run): 시트를 골라 테스트 수행 만들기 (v1.4.0.0, SYM-37/38/40)
테스트 수행은 프로젝트 전체 TC 를 담았고 시트를 고를 수 없었다.

- 생성 모달에 "포함할 시트" 추가. 기본 전체 선택, 체크 해제로 줄인다
- 고른 범위를 test_runs.sheet_names 에 저장한다. 생성 시점 필터가 아니라
  수행의 범위라서, 진행 중 수행이 새 TC 를 흡수할 때도 같은 조건을 건다
- 복제하면 범위도 따라간다. 폴더와 없는 시트는 받지 않고, 범위 밖 TC 의
  결과 제출은 400 으로 거부한다
- 시트 이름을 바꾸거나 지우면 그 시트를 담은 수행의 범위도 함께 고친다.
  이름만 바뀌어도 그 수행은 결과 저장이 전부 막혔다
- 대시보드 분모를 수행이 담은 TC 수로 바꿨다. 분자도 같은 기준으로 좁혀
  지운 TC 의 결과가 남지 않는다 (SYM-38)
- 결과 저장이 거부되면 서버가 준 사유를 띄우고 화면을 되돌린다 (SYM-40)
- 테스트 23건 추가. 백엔드 278건, 프론트 432건 통과

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01U8QHoWTN4U8F5QVZ7RJPVU
</commit_message>
<xml_diff>
--- a/Issue_list.xlsx
+++ b/Issue_list.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U150"/>
+  <dimension ref="A1:U154"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -11362,6 +11362,445 @@
         </is>
       </c>
     </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>ENH-046</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>enhancement</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>major</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>frontend</t>
+        </is>
+      </c>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>테스트 수행을 시트 단위로 만들 수 없다</t>
+        </is>
+      </c>
+      <c r="G151" t="inlineStr">
+        <is>
+          <t>- 새 테스트 수행을 만들면 프로젝트의 모든 TC 가 담긴다.
+- 담을 시트를 고르는 수단이 없다. 만든 뒤에는 시트 탭으로 보기만 걸러진다.</t>
+        </is>
+      </c>
+      <c r="H151" t="inlineStr">
+        <is>
+          <t>- 생성 모달에서 담을 시트를 고른다. 처음에는 전부 선택돼 있고 체크를 풀어 줄인다.
+- 고른 시트의 TC 만 수행에 담긴다.
+- 고른 범위가 수행에 저장되어, 진행 중 수행이 새 TC 를 흡수할 때도 그 범위를 지킨다.
+- 수행 상세의 시트 탭은 그 수행의 범위만 보여 준다.</t>
+        </is>
+      </c>
+      <c r="K151" t="inlineStr">
+        <is>
+          <t>- [x] 생성 모달에서 시트를 고를 수 있다. 기본은 전체 선택이고 체크 해제로 줄인다.
+- [x] 전부 해제하면 생성할 수 없다.
+- [x] 고른 시트의 TC 만 결과 행으로 만들어진다.
+- [x] 범위를 수행에 저장하고, 새 TC 흡수 시에도 지킨다.
+- [x] 수행을 복제하면 범위도 따라간다.
+- [x] 폴더와 없는 시트는 범위로 받지 않는다.
+- [x] 범위 밖 TC 의 결과 제출을 거부한다.
+- [x] 시트 탭이 그 수행의 범위만 보여 준다.
+- [x] 사용자 매뉴얼 갱신.</t>
+        </is>
+      </c>
+      <c r="N151" t="inlineStr">
+        <is>
+          <t>- 시트가 여러 개인 프로젝트에서 한 영역만 회귀 돌릴 때, 전체 TC 가 담긴 수행에서 다른 시트가 계속 미실행으로 남아 진행률이 실제와 다르게 보인다.
+- 라운드를 영역별로 나눠 돌리는 운영을 지금 방식으로는 표현할 수 없다.</t>
+        </is>
+      </c>
+      <c r="O151" t="inlineStr">
+        <is>
+          <t>- 생성 모달에 시트 체크박스를 넣고, 고른 시트를 test_runs.sheet_names (JSON, nullable) 에 저장한다. NULL 은 프로젝트 전체를 뜻해 기존 수행과 동작이 같다.
+- 생성 시점의 필터가 아니라 수행의 범위로 다룬다. run_sync_service.sync_run_results 에서도 같은 조건을 건다. 걸지 않으면 TC 하나가 생기는 순간 제외한 시트가 통째로 들어온다(재현 테스트로 확인).
+- QA 교차검증에서 나온 우회 경로 3건을 같이 막았다. 결과 제출(submit_results)이 시트 범위를 안 봐서 API 한 번으로 범위 밖 TC 가 들어오던 것, 폴더를 범위로 지정할 수 있던 것, 중복 시트명이 그대로 저장되던 것.
+- 시트 탭이 트리 루트만 보고 있어 폴더 밑 시트로 범위를 잡으면 탭이 하나도 안 나오던 것도 고쳤다.
+- 2차 QA 교차검증 대응: 시트 이름을 바꾸면 런 범위가 아무것도 가리키지 않게 되어 그 수행의 결과 저장이 전부 거부되고 새 TC 도 흡수되지 않던 것을 고쳤다(rename 과 같은 트랜잭션에서 범위도 치환). 시트 삭제 시에도 범위에서 뺀다. 이때 범위가 빌 수 있어 '없음' 과 '전체' 를 is not None 으로 갈랐다. 빈 목록이 falsy 로 떨어지면 담을 것이 없어진 수행이 프로젝트 전체를 담는다.</t>
+        </is>
+      </c>
+      <c r="P151" t="inlineStr">
+        <is>
+          <t>- backend/test_run_sheet_scope.py 10건. 범위 적용, 미지정 시 전체, 신규 TC 흡수의 범위 유지, 복제 승계, 폴더 거부, 없는 시트 400, 빈 목록 400, 중복 제거, 범위 밖 결과 제출 거부, 대시보드 분모.
+- frontend/src/test/TestRunSheetScope.test.tsx 7건.
+- 회귀 체크리스트 TC-TR-038, TC-TR-039 추가.
+- 동기화 가드와 페이로드 전달을 각각 되돌려 테스트가 실제로 실패하는지 확인했다.
+- 하지 않을 것: 이미 만든 수행의 범위를 나중에 바꾸는 기능, 테스트 플랜과의 연동.
+- 2차: 시트 rename 후 범위 유지, 삭제된 TC 결과의 대시보드 분자 제외 테스트 2건 추가(총 12건).</t>
+        </is>
+      </c>
+      <c r="Q151" t="inlineStr">
+        <is>
+          <t>- 테스트 수행 생성/복제/결과 제출, 수행 상세의 시트 탭.
+- test_runs 테이블에 컬럼 1개 추가.
+- 사용자 매뉴얼 8-1 절.</t>
+        </is>
+      </c>
+      <c r="R151" t="inlineStr">
+        <is>
+          <t>FE 1.3.3.0</t>
+        </is>
+      </c>
+      <c r="S151" t="inlineStr">
+        <is>
+          <t>FE 1.4.0.0 / BE 1.4.0.0 / DB 0.8.0.0</t>
+        </is>
+      </c>
+      <c r="T151" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="U151" t="inlineStr">
+        <is>
+          <t>SYM-37</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>BUG-091</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>bug</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>major</t>
+        </is>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>backend</t>
+        </is>
+      </c>
+      <c r="F152" t="inlineStr">
+        <is>
+          <t>대시보드가 프로젝트 전체 TC 를 분모로 써서 일부 시트만 담은 수행의 진행률이 틀리다</t>
+        </is>
+      </c>
+      <c r="G152" t="inlineStr">
+        <is>
+          <t>- 일부 시트만 담은 테스트 수행을 대시보드에서 고르면 총 건수가 그 수행이 담은 TC 수가 아니라 프로젝트 전체 TC 수로 나온다.
+- 그 수행의 TC 를 전부 PASS 로 입력해도 진행률이 100% 에 닿지 않고 미실행이 남는다.</t>
+        </is>
+      </c>
+      <c r="H152" t="inlineStr">
+        <is>
+          <t>- 수행을 골랐을 때 총 건수는 그 수행이 담은 TC 수다.
+- 그 수행을 전부 수행하면 진행률 100%, 미실행 0 이다.</t>
+        </is>
+      </c>
+      <c r="I152" t="inlineStr">
+        <is>
+          <t>- 결제 시트 4건을 전부 PASS 했는데 total 11, not_started 7, pass_rate 36.4 로 나왔다.</t>
+        </is>
+      </c>
+      <c r="J152" t="inlineStr">
+        <is>
+          <t>- 시트가 여러 개인 프로젝트에 일부 시트만 담은 테스트 수행이 있다.</t>
+        </is>
+      </c>
+      <c r="K152" t="inlineStr">
+        <is>
+          <t>1. 시트 3개짜리 프로젝트에서 시트 하나만 골라 테스트 수행을 만든다.
+2. 그 수행의 TC 를 전부 PASS 로 입력한다.
+3. 대시보드에서 그 수행을 고른다.</t>
+        </is>
+      </c>
+      <c r="L152" t="inlineStr">
+        <is>
+          <t>- 항상</t>
+        </is>
+      </c>
+      <c r="M152" t="inlineStr">
+        <is>
+          <t>- 실측 2026-09-08, GET /api/projects/{id}/dashboard/summary?run_id={run} 응답:
+  {"total": 11, "pass": 4, "not_started": 7, "pass_rate": 36.4}
+- dashboard.py 의 total 은 TestCase 를 project_id 로만 세고, run_id 분기는 그 값을 그대로 분모로 쓴다.
+- priority, category, rounds, overview 도 같은 방식이다.</t>
+        </is>
+      </c>
+      <c r="N152" t="inlineStr">
+        <is>
+          <t>- 코드 리뷰 (SYM-37 시트 범위 기능 QA 교차검증)</t>
+        </is>
+      </c>
+      <c r="O152" t="inlineStr">
+        <is>
+          <t>원인: 대시보드가 총 건수를 TestCase 에서 project_id 로만 세고, run_id 분기는 그 값을 그대로 분모로 썼다. 시트 범위 기능이 생기기 전에는 프로젝트 전체 TC 수와 수행이 담은 TC 수가 항상 같아서 드러나지 않았다.
+수정: run_id 가 오면 그 수행의 결과 행에 들어 있는 TC 로 총계를 좁힌다. summary, priority, category 에 적용했고, rounds 는 라운드별 대표 수행의 결과 행 수를 분모로 쓴다. 전역 개요는 최신 수행이 담은 행 수를 분모로 쓴다(수치가 그 수행에서 나오므로 분모도 같아야 한다).
+- 2차 QA 대응: summary 와 rounds 의 분자도 활성 TC 로 좁혔다. 분모만 좁히면 지운 TC 의 결과가 남아 pass 가 total 을 넘는다. rounds 와 전역 개요에서 결과 행이 0 인 런이 프로젝트 전체로 되돌아가던 fallback 도 고쳤다.</t>
+        </is>
+      </c>
+      <c r="P152" t="inlineStr">
+        <is>
+          <t>- backend/test_run_sheet_scope.py 의 대시보드 테스트 1건. summary, category, priority 를 함께 본다.
+- 회귀 체크리스트 TC-TR-040 추가.
+- 수정을 되돌려 테스트가 실패하는지 확인했다.
+- reports.py 와 testplans.py 는 TestResult 행 수를 직접 세는 방식이라 손대지 않았다.</t>
+        </is>
+      </c>
+      <c r="Q152" t="inlineStr">
+        <is>
+          <t>- 대시보드 summary, priority, category, rounds 와 전역 개요.
+- 일부 시트만 담은 수행의 수치가 달라진다(실측 36.4% -&gt; 100%).</t>
+        </is>
+      </c>
+      <c r="R152" t="inlineStr">
+        <is>
+          <t>BE 1.3.3.0</t>
+        </is>
+      </c>
+      <c r="S152" t="inlineStr">
+        <is>
+          <t>BE 1.4.0.0</t>
+        </is>
+      </c>
+      <c r="T152" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="U152" t="inlineStr">
+        <is>
+          <t>SYM-38</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>BUG-092</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>bug</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>major</t>
+        </is>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>db</t>
+        </is>
+      </c>
+      <c r="F153" t="inlineStr">
+        <is>
+          <t>pre-Alembic DB 를 stamp(head) 로만 처리해 새 컬럼이 없는 채로 최신 버전이 된다</t>
+        </is>
+      </c>
+      <c r="G153" t="inlineStr">
+        <is>
+          <t>- 테이블은 있는데 alembic_version 테이블이 없는 DB 를 만나면 main.py 의 lifespan 이 stamp(head) 만 한다.
+- 실제 스키마는 그대로인데 버전만 최신으로 찍혀, 이후 어떤 마이그레이션도 적용되지 않는다.</t>
+        </is>
+      </c>
+      <c r="H153" t="inlineStr">
+        <is>
+          <t>- 스키마와 alembic 버전이 어긋나지 않는다. 또는 어긋난 것을 감지해 기동을 멈추고 알린다.</t>
+        </is>
+      </c>
+      <c r="I153" t="inlineStr">
+        <is>
+          <t>- 이후 ORM 이 새 컬럼(예: test_runs.sheet_names)을 조회하면 no such column 으로 실패한다.</t>
+        </is>
+      </c>
+      <c r="J153" t="inlineStr">
+        <is>
+          <t>- Alembic 도입(v1.2.1.0) 이전에 만들어져 계속 쓰이는 DB 파일.</t>
+        </is>
+      </c>
+      <c r="K153" t="inlineStr">
+        <is>
+          <t>1. alembic_version 테이블이 없고 다른 테이블은 있는 tc_manager.db 를 준비한다.
+2. 서버를 기동한다.
+3. sqlite 로 test_runs 스키마를 확인한다.</t>
+        </is>
+      </c>
+      <c r="L153" t="inlineStr">
+        <is>
+          <t>- 미확인</t>
+        </is>
+      </c>
+      <c r="M153" t="inlineStr">
+        <is>
+          <t>- backend/main.py 의 lifespan: tables and "alembic_version" not in tables 이면 alembic_command.stamp(cfg, "head") 만 부른다.
+- 이 경로에는 컬럼을 만드는 단계가 없다.</t>
+        </is>
+      </c>
+      <c r="N153" t="inlineStr">
+        <is>
+          <t>- 코드 리뷰 (SYM-37 QA 교차검증, Codex)</t>
+        </is>
+      </c>
+      <c r="R153" t="inlineStr">
+        <is>
+          <t>BE 1.3.3.0</t>
+        </is>
+      </c>
+      <c r="T153" t="inlineStr">
+        <is>
+          <t>미해결</t>
+        </is>
+      </c>
+      <c r="U153" t="inlineStr">
+        <is>
+          <t>SYM-39</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>BUG-093</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>bug</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>major</t>
+        </is>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>frontend</t>
+        </is>
+      </c>
+      <c r="F154" t="inlineStr">
+        <is>
+          <t>테스트 수행에서 결과 저장이 거부돼도 이유를 알 수 없고 화면 값이 그대로 남는다</t>
+        </is>
+      </c>
+      <c r="G154" t="inlineStr">
+        <is>
+          <t>- 결과 저장이 서버에서 거부되면 이유와 무관하게 '저장 실패' 만 뜬다.
+- 화면의 셀 값은 바뀐 채로 남아 저장된 것처럼 보인다. 새로고침하면 서버 값으로 돌아간다.</t>
+        </is>
+      </c>
+      <c r="H154" t="inlineStr">
+        <is>
+          <t>- 서버가 준 거부 사유를 그대로 보여 준다.
+- 거부된 값은 화면에서도 서버 값으로 되돌아간다.</t>
+        </is>
+      </c>
+      <c r="I154" t="inlineStr">
+        <is>
+          <t>- catch 블록이 예외를 버리고 고정 문구만 띄운다.
+- 되돌리는 코드가 없어 화면과 DB 가 갈라진다.</t>
+        </is>
+      </c>
+      <c r="J154" t="inlineStr">
+        <is>
+          <t>- 결과 저장이 거부되는 상황. 시트 범위 밖 TC 제출이 이번에 새로 생긴 거부 경로다.</t>
+        </is>
+      </c>
+      <c r="K154" t="inlineStr">
+        <is>
+          <t>1. 시트를 골라 테스트 수행을 만든다.
+2. 범위 밖 TC 의 결과를 저장하는 요청이 나가게 한다.
+3. 화면의 값과 서버 값을 대조한다.</t>
+        </is>
+      </c>
+      <c r="L154" t="inlineStr">
+        <is>
+          <t>- 항상</t>
+        </is>
+      </c>
+      <c r="M154" t="inlineStr">
+        <is>
+          <t>- TestRunManager.tsx 의 saveOneResult, saveManyResults 가 catch 에서 toast.error(t('saveFailed')) 만 부른다.
+- 같은 레포 ProjectSettings.tsx 는 err.response.data.detail 을 꺼내 쓴다. 패턴이 갈려 있다.
+- SYM-35 가 TC 관리 그리드에서 같은 유형으로 이미 한 번 났다.</t>
+        </is>
+      </c>
+      <c r="N154" t="inlineStr">
+        <is>
+          <t>- 코드 리뷰 (SYM-37 QA 교차검증 2차)</t>
+        </is>
+      </c>
+      <c r="O154" t="inlineStr">
+        <is>
+          <t>원인: saveOneResult 와 saveManyResults 의 catch 가 예외를 버리고 고정 문구만 띄웠다. 되돌리는 코드도 없어 거부된 값이 화면에 남았다.
+수정: 공용 handleSaveError 로 모아 서버가 준 detail 을 그대로 띄우고, 실패하면 런 상세를 다시 받아 화면을 서버 값으로 되돌린다.</t>
+        </is>
+      </c>
+      <c r="P154" t="inlineStr">
+        <is>
+          <t>- frontend/src/test/TestRunSaveError.test.tsx 4건. ag-grid 를 자체 모킹해 onCellValueChanged 저장 경로를 실제로 태운다. detail 노출, 실패 시 재조회, detail 이 없을 때 기본 문구, 성공 시 재조회 안 함.
+- 옛 처리로 되돌려 2건이 실패하는지 확인했다.
+- 하지 않을 것: 셀 단위 롤백은 넣지 않았다. 런 상세를 다시 받는 편이 경로가 하나라 어긋날 여지가 적다.</t>
+        </is>
+      </c>
+      <c r="Q154" t="inlineStr">
+        <is>
+          <t>- 테스트 수행 그리드의 결과/실제결과/이슈링크/비고 저장 실패 처리 전체.</t>
+        </is>
+      </c>
+      <c r="R154" t="inlineStr">
+        <is>
+          <t>FE 1.3.3.0</t>
+        </is>
+      </c>
+      <c r="S154" t="inlineStr">
+        <is>
+          <t>FE 1.4.0.0</t>
+        </is>
+      </c>
+      <c r="T154" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="U154" t="inlineStr">
+        <is>
+          <t>SYM-40</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix(run): 수행 화면과 엑셀의 No 를 목록 순번으로 통일 (v1.4.1.0, SYM-41~44)
시트를 골라 만든 수행의 No 가 1 이 아니라 4, 5, 6, 51 로 시작했다.

- 재번호가 "전체" 탭 경로에만 있었다. 기본 탭은 첫 시트고 시트를 골라 만든
  수행은 전체 탭이 없어, 실제로 보게 되는 화면은 대부분 재번호 없는 쪽이었다
- 시트 탭과 전체 탭을 한 경로로 합쳐 항상 1 부터 매긴다. 시트 순서와 기본 탭도
  트리 루트가 아니라 펴 놓은 잎 시트에서 고른다
- 저장된 no 에 구멍을 낸 것은 복제였다. 신규 행 추가와 임포트는 시트 기준으로
  번호를 붙이는데 복제만 프로젝트 전체 max(no)+1 을 줬다. 시트 기준으로 바꾸고,
  지운 TC 가 쥐고 있던 번호는 복원할 때 겹치므로 쓰지 않는다
- 수행 엑셀과 리포트 엑셀이 services/sheet_order.py 로 같은 차례와 번호를 낸다.
  한쪽만 고치면 같은 행이 두 파일에서 다른 번호를 단다
- 수행 이름에 한글이 있으면 내보내기가 500 이었다. 헤더는 latin-1 만 담는다.
  나머지 내보내기 3곳이 쓰던 RFC 5987 로 맞췄다
- 테스트 15건 추가. 백엔드 287건, 프론트 440건 통과

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016UKFCyy7maLAXe6Si7ZiqR
</commit_message>
<xml_diff>
--- a/Issue_list.xlsx
+++ b/Issue_list.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U154"/>
+  <dimension ref="A1:U162"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -11801,6 +11801,776 @@
         </is>
       </c>
     </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>BUG-094</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>bug</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>major</t>
+        </is>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>frontend</t>
+        </is>
+      </c>
+      <c r="F155" t="inlineStr">
+        <is>
+          <t>시트를 골라 만든 테스트 수행의 No 가 1 부터 시작하지 않는다</t>
+        </is>
+      </c>
+      <c r="G155" t="inlineStr">
+        <is>
+          <t>- 시트를 골라 만든 수행을 열면 No 컬럼이 4, 5, 6, 51 처럼 나온다
+- 시트가 둘 이상인 프로젝트의 수행도 기본 탭(첫 시트)에서 같은 증상이 난다</t>
+        </is>
+      </c>
+      <c r="H155" t="inlineStr">
+        <is>
+          <t>- No 는 지금 보고 있는 목록의 순번이라 1 부터 이어져야 한다</t>
+        </is>
+      </c>
+      <c r="I155" t="inlineStr">
+        <is>
+          <t>- TC 에 저장된 no 가 그대로 나온다. 프로젝트 118 의 수행 34(결제 시트)에서 4, 5, 6, 51</t>
+        </is>
+      </c>
+      <c r="K155" t="inlineStr">
+        <is>
+          <t>1. 시트가 둘 이상인 프로젝트에서 시트 하나만 골라 수행을 만든다
+2. 그 수행을 연다
+3. No 컬럼을 본다</t>
+        </is>
+      </c>
+      <c r="L155" t="inlineStr">
+        <is>
+          <t>- 항상</t>
+        </is>
+      </c>
+      <c r="M155" t="inlineStr">
+        <is>
+          <t>- 실 DB 조회: 수행 34 의 TC no 가 4, 5, 6, 51
+- 브라우저 실측: No 컬럼 값이 4, 5, 6, 51</t>
+        </is>
+      </c>
+      <c r="N155" t="inlineStr">
+        <is>
+          <t>- 사용자</t>
+        </is>
+      </c>
+      <c r="O155" t="inlineStr">
+        <is>
+          <t>원인: - TestRunManager.tsx 의 loadRunDetail 이 재번호를 '전체' 탭 경로에서만 한다
+- 시트가 둘 이상이면 기본 탭이 첫 시트이고, 시트를 골라 만든 수행은 전체 탭 자체가 없다. 실제로 보게 되는 화면이 대부분 재번호 없는 쪽이었다
+- 전체 탭 분기의 조건도 트리 루트 개수라, 시트를 폴더 하나에 모아 둔 프로젝트는 전체 탭에서도 재번호가 걸리지 않았다
+수정 내용: - 시트 탭과 전체 탭을 한 경로로 합쳐 항상 1 부터 매긴다
+- 시트 순서를 트리 루트가 아니라 펴 놓은 잎 시트에서 가져온다
+- 기본 탭도 잎 시트로 고른다. 루트 첫 칸이 폴더면 폴더 이름으로 걸러 그리드가 빈 채로 열리고 상세를 두 번 받았다
+- 서버가 준 객체를 제자리에서 고치지 않고 새 객체로 바꿔 저장된 no 를 건드리지 않는다</t>
+        </is>
+      </c>
+      <c r="P155" t="inlineStr">
+        <is>
+          <t>- TestRunNumbering.test.tsx 8건. 시트 범위 수행, 시트 탭, 폴더로 묶은 프로젝트, 시트 목록이 늦게 오는 경우, 저장된 no 불변까지 본다
+- 번호만 보면 시트 순서가 틀려도 1,2,3,4 로 보이므로 TC ID 순서도 함께 단언한다</t>
+        </is>
+      </c>
+      <c r="Q155" t="inlineStr">
+        <is>
+          <t>- 테스트 수행 화면의 No 컬럼</t>
+        </is>
+      </c>
+      <c r="R155" t="inlineStr">
+        <is>
+          <t>FE 1.4.0.0</t>
+        </is>
+      </c>
+      <c r="S155" t="inlineStr">
+        <is>
+          <t>FE 1.4.1.0</t>
+        </is>
+      </c>
+      <c r="T155" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="U155" t="inlineStr">
+        <is>
+          <t>SYM-41</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>BUG-095</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>bug</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>major</t>
+        </is>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>backend</t>
+        </is>
+      </c>
+      <c r="F156" t="inlineStr">
+        <is>
+          <t>TC 복제가 프로젝트 전체 max(no)+1 을 줘서 시트 안 번호에 구멍이 난다</t>
+        </is>
+      </c>
+      <c r="G156" t="inlineStr">
+        <is>
+          <t>- 시트 안에서 1 부터 이어지던 번호가 복제 뒤 갑자기 다른 시트의 최대값 다음으로 뛴다
+- 프로젝트 118 의 결제 시트: 1, 2, 3 다음 복제본이 51</t>
+        </is>
+      </c>
+      <c r="H156" t="inlineStr">
+        <is>
+          <t>- no 는 시트 안 순번이다. 결제 시트의 최대가 3 이면 복제본은 4 여야 한다</t>
+        </is>
+      </c>
+      <c r="I156" t="inlineStr">
+        <is>
+          <t>- 다른 시트(로그인, 최대 50)의 번호가 따라와 51 이 붙었다</t>
+        </is>
+      </c>
+      <c r="K156" t="inlineStr">
+        <is>
+          <t>1. 시트 둘을 만들고 각각 no 를 1 부터 매긴다
+2. 번호가 작은 쪽 시트의 TC 를 복제한다
+3. 새 TC 의 no 를 본다</t>
+        </is>
+      </c>
+      <c r="L156" t="inlineStr">
+        <is>
+          <t>- 항상</t>
+        </is>
+      </c>
+      <c r="M156" t="inlineStr">
+        <is>
+          <t>- 실 DB: 프로젝트 118 결제 시트에 no 4, 5, 6, 51
+- 재현 테스트에서 결제 시트 복제본이 4 가 아니라 501</t>
+        </is>
+      </c>
+      <c r="N156" t="inlineStr">
+        <is>
+          <t>- 코드 리뷰</t>
+        </is>
+      </c>
+      <c r="O156" t="inlineStr">
+        <is>
+          <t>원인: - testcases.py 의 clone 과 bulk-clone 이 max(no) 를 프로젝트 전체에서 구했다
+- 신규 행 추가(프론트가 그 시트의 max+1 을 보낸다)와 엑셀 임포트(no_offset=0)는 시트 기준이라 복제만 규약을 어겼다
+수정 내용: - _max_no_in_sheet 헬퍼를 두고 두 복제 경로가 시트 기준 max+1 을 쓰게 했다
+- bulk-clone 은 시트별 카운터를 캐시해 같은 시트 다건 복제에서 번호가 겹치지 않는다
+- max 를 구할 때 지운 TC 도 센다. 삭제는 soft delete 라, 살아 있는 것만 보면 지운 번호를 복제가 다시 쓰고 복원하는 순간 같은 시트에 같은 번호가 둘이 된다</t>
+        </is>
+      </c>
+      <c r="P156" t="inlineStr">
+        <is>
+          <t>- test_tc_clone_numbering.py 5건. 단건/일괄 복제, 다른 시트의 큰 번호 무시, 지운 TC 번호 재사용 금지까지 본다</t>
+        </is>
+      </c>
+      <c r="Q156" t="inlineStr">
+        <is>
+          <t>- TC 복제로 만들어지는 새 TC 의 no. 이미 만들어진 TC 는 그대로다</t>
+        </is>
+      </c>
+      <c r="R156" t="inlineStr">
+        <is>
+          <t>BE 1.4.0.0</t>
+        </is>
+      </c>
+      <c r="S156" t="inlineStr">
+        <is>
+          <t>BE 1.4.1.0</t>
+        </is>
+      </c>
+      <c r="T156" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="U156" t="inlineStr">
+        <is>
+          <t>SYM-42</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>BUG-096</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>bug</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>major</t>
+        </is>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>backend</t>
+        </is>
+      </c>
+      <c r="F157" t="inlineStr">
+        <is>
+          <t>수행 이름에 한글이 있으면 엑셀 내보내기가 500 이다</t>
+        </is>
+      </c>
+      <c r="G157" t="inlineStr">
+        <is>
+          <t>- 테스트 수행 화면의 Excel 버튼이 실패한다</t>
+        </is>
+      </c>
+      <c r="H157" t="inlineStr">
+        <is>
+          <t>- 이름과 무관하게 파일이 내려와야 한다</t>
+        </is>
+      </c>
+      <c r="I157" t="inlineStr">
+        <is>
+          <t>- 500 Internal server error. 같은 수행을 영문 이름으로 만들면 200</t>
+        </is>
+      </c>
+      <c r="K157" t="inlineStr">
+        <is>
+          <t>1. 이름에 한글이 든 테스트 수행을 만든다
+2. 그 수행에서 Excel 을 누른다</t>
+        </is>
+      </c>
+      <c r="L157" t="inlineStr">
+        <is>
+          <t>- 항상</t>
+        </is>
+      </c>
+      <c r="M157" t="inlineStr">
+        <is>
+          <t>- 같은 프로젝트에서 ASCII 이름 200, 한글 이름 500 을 나란히 실측</t>
+        </is>
+      </c>
+      <c r="N157" t="inlineStr">
+        <is>
+          <t>- 코드 리뷰</t>
+        </is>
+      </c>
+      <c r="O157" t="inlineStr">
+        <is>
+          <t>원인: - testruns.py 의 내보내기가 Content-Disposition 에 수행 이름을 그대로 넣었다. 헤더는 latin-1 만 담아서 인코딩에서 터진다
+- 리포트와 TC 목록 내보내기 3곳은 이미 RFC 5987 을 쓰고 있었고 이 한 곳만 옛 방식이었다
+수정 내용: - filename*=UTF-8'' 형식으로 맞췄다. 나머지 내보내기와 같은 모양이다</t>
+        </is>
+      </c>
+      <c r="P157" t="inlineStr">
+        <is>
+          <t>- test_run_export_numbering.py 가 한글 이름 수행으로 내보내기를 호출한다. 500 이면 그 자리에서 걸린다</t>
+        </is>
+      </c>
+      <c r="Q157" t="inlineStr">
+        <is>
+          <t>- 테스트 수행 엑셀 내보내기</t>
+        </is>
+      </c>
+      <c r="R157" t="inlineStr">
+        <is>
+          <t>BE 1.4.0.0</t>
+        </is>
+      </c>
+      <c r="S157" t="inlineStr">
+        <is>
+          <t>BE 1.4.1.0</t>
+        </is>
+      </c>
+      <c r="T157" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="U157" t="inlineStr">
+        <is>
+          <t>SYM-43</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>BUG-097</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>bug</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>minor</t>
+        </is>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>backend</t>
+        </is>
+      </c>
+      <c r="F158" t="inlineStr">
+        <is>
+          <t>같은 수행인데 수행 엑셀과 리포트 엑셀의 No 와 행 순서가 다르다</t>
+        </is>
+      </c>
+      <c r="G158" t="inlineStr">
+        <is>
+          <t>- 한 수행을 두 곳에서 엑셀로 뽑으면 같은 행이 서로 다른 번호를 단다
+- 여러 시트를 담은 수행에서는 행 순서도 다르다</t>
+        </is>
+      </c>
+      <c r="H158" t="inlineStr">
+        <is>
+          <t>- 같은 수행이면 두 파일의 번호와 순서가 같아야 한다</t>
+        </is>
+      </c>
+      <c r="I158" t="inlineStr">
+        <is>
+          <t>- 수행 엑셀은 1, 2, 3, 4. 리포트 엑셀은 저장된 no 를 그대로 써서 4, 5, 6, 51</t>
+        </is>
+      </c>
+      <c r="K158" t="inlineStr">
+        <is>
+          <t>1. 시트가 여럿인 프로젝트에서 수행을 만든다
+2. 테스트 수행 화면에서 Excel 을 받는다
+3. 리포트 화면에서 엑셀을 받는다
+4. 두 파일의 No 컬럼을 대조한다</t>
+        </is>
+      </c>
+      <c r="L158" t="inlineStr">
+        <is>
+          <t>- 항상</t>
+        </is>
+      </c>
+      <c r="M158" t="inlineStr">
+        <is>
+          <t>- 두 응답을 같은 수행으로 받아 행 단위로 대조한 테스트가 첫 행부터 어긋났다</t>
+        </is>
+      </c>
+      <c r="N158" t="inlineStr">
+        <is>
+          <t>- 코드 리뷰</t>
+        </is>
+      </c>
+      <c r="O158" t="inlineStr">
+        <is>
+          <t>원인: - 두 내보내기가 정렬과 번호를 각자 들고 있었다. 수행 엑셀만 고치면서 갈라졌다
+수정 내용: - services/sheet_order.py 를 만들어 두 내보내기가 같은 함수로 세우고 같은 규약으로 번호를 매긴다
+- 시트 트리가 비어 있는 옛 데이터에서도 화면과 같은 차례가 되도록 폴백을 넣었다</t>
+        </is>
+      </c>
+      <c r="P158" t="inlineStr">
+        <is>
+          <t>- 두 응답을 행 단위로 대조하는 테스트를 뒀다. 한쪽만 고치면 실패한다
+- 화면 시트 탭 순서와 내보내기 순서가 같은지 보는 테스트도 함께 뒀다</t>
+        </is>
+      </c>
+      <c r="Q158" t="inlineStr">
+        <is>
+          <t>- 리포트 엑셀의 Results 시트</t>
+        </is>
+      </c>
+      <c r="R158" t="inlineStr">
+        <is>
+          <t>BE 1.4.0.0</t>
+        </is>
+      </c>
+      <c r="S158" t="inlineStr">
+        <is>
+          <t>BE 1.4.1.0</t>
+        </is>
+      </c>
+      <c r="T158" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="U158" t="inlineStr">
+        <is>
+          <t>SYM-44</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>BUG-098</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>bug</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>major</t>
+        </is>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>backend</t>
+        </is>
+      </c>
+      <c r="F159" t="inlineStr">
+        <is>
+          <t>라운드가 비어 있는 수행이 하나라도 있으면 그 프로젝트의 수행 목록이 500 이다</t>
+        </is>
+      </c>
+      <c r="G159" t="inlineStr">
+        <is>
+          <t>- 특정 프로젝트에서 테스트 수행 탭이 '등록된 테스트 수행이 없습니다' 로 보인다. DB 에는 수행이 있다</t>
+        </is>
+      </c>
+      <c r="H159" t="inlineStr">
+        <is>
+          <t>- 라운드가 비어 있어도 목록에 나와야 한다</t>
+        </is>
+      </c>
+      <c r="I159" t="inlineStr">
+        <is>
+          <t>- GET /api/projects/116/testruns 가 500. 화면은 빈 목록으로 그린다</t>
+        </is>
+      </c>
+      <c r="K159" t="inlineStr">
+        <is>
+          <t>1. round 가 NULL 인 수행이 있는 프로젝트를 연다
+2. 테스트 수행 탭을 누른다</t>
+        </is>
+      </c>
+      <c r="L159" t="inlineStr">
+        <is>
+          <t>- 항상</t>
+        </is>
+      </c>
+      <c r="M159" t="inlineStr">
+        <is>
+          <t>- 실 DB 프로젝트 116 에 round 가 NULL 인 수행 2건(25, 26)
+- 같은 서버에서 프로젝트 118 은 200, 116 은 500</t>
+        </is>
+      </c>
+      <c r="N159" t="inlineStr">
+        <is>
+          <t>- 코드 리뷰</t>
+        </is>
+      </c>
+      <c r="R159" t="inlineStr">
+        <is>
+          <t>BE 1.4.1.0</t>
+        </is>
+      </c>
+      <c r="T159" t="inlineStr">
+        <is>
+          <t>미해결</t>
+        </is>
+      </c>
+      <c r="U159" t="inlineStr">
+        <is>
+          <t>SYM-45</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>BUG-099</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>bug</t>
+        </is>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>major</t>
+        </is>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>db</t>
+        </is>
+      </c>
+      <c r="F160" t="inlineStr">
+        <is>
+          <t>기존 TC 의 no 가 시트 안 순번 규약을 만족하지 않는다</t>
+        </is>
+      </c>
+      <c r="G160" t="inlineStr">
+        <is>
+          <t>- 시트 안 번호에 구멍과 중복이 남아 있다. TC 관리 화면의 시트 탭과 TC 엑셀 내보내기에 그대로 보인다</t>
+        </is>
+      </c>
+      <c r="H160" t="inlineStr">
+        <is>
+          <t>- no 는 시트 안에서 1 부터 이어지는 순번이다</t>
+        </is>
+      </c>
+      <c r="I160" t="inlineStr">
+        <is>
+          <t>- 프로젝트 118 결제 시트가 4, 5, 6, 51. 프로젝트 116 은 시트별 최소값이 1, 28, 58, 80, 104, 117, 127, 131 로 흩어져 있고 최대값이 430 대까지 간다</t>
+        </is>
+      </c>
+      <c r="K160" t="inlineStr">
+        <is>
+          <t>1. TC 관리에서 번호가 흩어진 시트를 연다
+2. No 컬럼을 본다</t>
+        </is>
+      </c>
+      <c r="L160" t="inlineStr">
+        <is>
+          <t>- 항상</t>
+        </is>
+      </c>
+      <c r="M160" t="inlineStr">
+        <is>
+          <t>- 실 DB 시트별 min/max 조회 결과</t>
+        </is>
+      </c>
+      <c r="N160" t="inlineStr">
+        <is>
+          <t>- 코드 리뷰</t>
+        </is>
+      </c>
+      <c r="R160" t="inlineStr">
+        <is>
+          <t>BE 1.4.1.0</t>
+        </is>
+      </c>
+      <c r="T160" t="inlineStr">
+        <is>
+          <t>미해결</t>
+        </is>
+      </c>
+      <c r="U160" t="inlineStr">
+        <is>
+          <t>SYM-46</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>BUG-100</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>bug</t>
+        </is>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>minor</t>
+        </is>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>backend</t>
+        </is>
+      </c>
+      <c r="F161" t="inlineStr">
+        <is>
+          <t>동시에 복제하면 같은 시트에 같은 no 가 들어갈 수 있다</t>
+        </is>
+      </c>
+      <c r="G161" t="inlineStr">
+        <is>
+          <t>- 같은 시트의 TC 를 두 요청이 동시에 복제하면 둘 다 같은 번호를 받을 수 있다</t>
+        </is>
+      </c>
+      <c r="H161" t="inlineStr">
+        <is>
+          <t>- 시트 안에서 no 는 겹치지 않아야 한다</t>
+        </is>
+      </c>
+      <c r="I161" t="inlineStr">
+        <is>
+          <t>- 두 요청이 같은 max(no) 를 읽고 각자 +1 을 한다. no 에 유니크 제약이 없어 DB 도 막지 않는다</t>
+        </is>
+      </c>
+      <c r="K161" t="inlineStr">
+        <is>
+          <t>1. 같은 시트의 TC 두 건에 대해 복제 요청을 동시에 보낸다
+2. 두 새 TC 의 no 를 본다</t>
+        </is>
+      </c>
+      <c r="L161" t="inlineStr">
+        <is>
+          <t>- 미확인</t>
+        </is>
+      </c>
+      <c r="M161" t="inlineStr">
+        <is>
+          <t>- 코드 경로만 확인했다. 실제 충돌은 재현하지 않았다. testcases.py 의 두 복제 경로가 max 조회와 삽입 사이를 잠그지 않는다</t>
+        </is>
+      </c>
+      <c r="N161" t="inlineStr">
+        <is>
+          <t>- 코드 리뷰</t>
+        </is>
+      </c>
+      <c r="R161" t="inlineStr">
+        <is>
+          <t>BE 1.4.1.0</t>
+        </is>
+      </c>
+      <c r="T161" t="inlineStr">
+        <is>
+          <t>미해결</t>
+        </is>
+      </c>
+      <c r="U161" t="inlineStr">
+        <is>
+          <t>SYM-47</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>SEC-015</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>bug</t>
+        </is>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>minor</t>
+        </is>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>security</t>
+        </is>
+      </c>
+      <c r="F162" t="inlineStr">
+        <is>
+          <t>수행 엑셀과 리포트 엑셀에 수식 인젝션 새니타이즈가 없다</t>
+        </is>
+      </c>
+      <c r="G162" t="inlineStr">
+        <is>
+          <t>- TC 내용이 =, +, -, @ 로 시작하면 엑셀에서 수식으로 해석된다</t>
+        </is>
+      </c>
+      <c r="H162" t="inlineStr">
+        <is>
+          <t>- 세 내보내기 경로가 같은 새니타이즈를 거쳐야 한다</t>
+        </is>
+      </c>
+      <c r="I162" t="inlineStr">
+        <is>
+          <t>- TC 목록 내보내기(export_service.py)에만 새니타이즈가 있고 수행 엑셀과 리포트 엑셀에는 없다</t>
+        </is>
+      </c>
+      <c r="K162" t="inlineStr">
+        <is>
+          <t>1. 기대 결과 칸에 =1+1 로 시작하는 값을 넣는다
+2. 수행 엑셀을 받아 연다</t>
+        </is>
+      </c>
+      <c r="L162" t="inlineStr">
+        <is>
+          <t>- 미확인</t>
+        </is>
+      </c>
+      <c r="M162" t="inlineStr">
+        <is>
+          <t>- export_service.py 에 새니타이즈 함수가 있고 testruns.py, reports.py 에는 호출이 없다</t>
+        </is>
+      </c>
+      <c r="N162" t="inlineStr">
+        <is>
+          <t>- 코드 리뷰</t>
+        </is>
+      </c>
+      <c r="R162" t="inlineStr">
+        <is>
+          <t>BE 1.4.1.0</t>
+        </is>
+      </c>
+      <c r="T162" t="inlineStr">
+        <is>
+          <t>미해결</t>
+        </is>
+      </c>
+      <c r="U162" t="inlineStr">
+        <is>
+          <t>SYM-48</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
refactor(tc): TC 번호 관리를 서버와 DB 제약으로 (v1.5.0.0, SYM-45~50)
앞 커밋이 수행 화면의 No 를 목록 순번으로 바꿨다. 그런데 저장된 no 자체는
여전히 아무나 정할 수 있었고, 마이그레이션으로 한 번 정리해도 다음 임포트
한 번에 되돌아가는 상태였다.

- no 는 살아 있는 TC 의 시트 안 순번이다. (project_id, sheet_name, no)
  부분 유니크 인덱스로 DB 가 강제한다. 기존 데이터는 시트마다 1..N 으로 다시
  매겼다. 실 DB 23개 시트 중 13개가 규약을 어기고 있었다
- 번호를 넣는 네 경로를 서버가 통제한다. 신규 생성과 수정은 보낸 값을 쓰지
  않고, 임포트 세 종류는 파일의 No 를 차례로만 쓰고, 정렬은 한 시트 전체를
  1..N 으로 보낼 때만 받는다
- 번호를 옮기는 곳은 모두 한 번 비켜 둔 뒤 최종 값을 쓴다. 유니크 인덱스는
  행 단위로 검사해서, 자리를 맞바꾸는 도중에 겹치면 그 자리에서 터진다
- 라운드가 비어 있으면 그 프로젝트의 수행 목록 전체가 500 이었다. 컬럼을
  NOT NULL 로 바꾸고 2건을 채웠다. 쓰기 쪽도 400 으로 거절한다
- 수행 엑셀과 리포트 엑셀에 수식 인젝션 방어가 없었다. 세 내보내기가 같은
  함수를 쓴다
- 테스트 건너뛰기 판정이 포트 기준이라 CI 에서 40건이 한 줄도 안 돌고 있었다.
  격리 여부로 바꿨다. 기본 조건 수집이 262건에서 332건이 됐다
- 테스트 45건 추가. 백엔드 332건, 프론트 445건 통과

자리 판정: 번호 관리 책임을 코드 규율에서 서버와 DB 제약으로 옮긴 구조
변경이라 B(feature) 로 본다.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016UKFCyy7maLAXe6Si7ZiqR
</commit_message>
<xml_diff>
--- a/Issue_list.xlsx
+++ b/Issue_list.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U162"/>
+  <dimension ref="A1:U164"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -12306,14 +12306,37 @@
           <t>- 코드 리뷰</t>
         </is>
       </c>
+      <c r="O159" t="inlineStr">
+        <is>
+          <t>원인: * 응답 스키마가 `round` 를 필수 정수로 읽는데 컬럼은 NULL 을 받았다. 목록 응답 하나가 못 만들어지면 그 프로젝트의 수행 목록 전체가 500 이 된다.
+수정 내용: * 컬럼을 NOT NULL, server_default 1 로 바꾸고 비어 있던 2건을 1 라운드로 채웠다 (alembic e5a83f21c760)
+* 응답 스키마도 옛 NULL 을 1 로 읽어 마이그레이션 전 DB 를 보는 서버에서 다시 터지지 않게 했다
+* 쓰기 쪽도 막았다. `PUT /testruns` 에 `round: null` 을 보내면 400 으로 거절한다. 전에는 커밋에서 제약에 걸려 409 가 났고 이유를 알 수 없었다</t>
+        </is>
+      </c>
+      <c r="P159" t="inlineStr">
+        <is>
+          <t>* `test_run_round_nullable.py` 4건. 컬럼 제약, 실제 쓰기 거부, 수정 API 거절, 옛 NULL 읽기까지 본다</t>
+        </is>
+      </c>
+      <c r="Q159" t="inlineStr">
+        <is>
+          <t>* 테스트 수행 목록 API. 실 DB 프로젝트 116 이 열리지 않던 것이 정상으로 돌아왔다</t>
+        </is>
+      </c>
       <c r="R159" t="inlineStr">
         <is>
           <t>BE 1.4.1.0</t>
         </is>
       </c>
+      <c r="S159" t="inlineStr">
+        <is>
+          <t>* BE 1.4.2.0 / DB 0.8.1.0</t>
+        </is>
+      </c>
       <c r="T159" t="inlineStr">
         <is>
-          <t>미해결</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="U159" t="inlineStr">
@@ -12389,14 +12412,40 @@
           <t>- 코드 리뷰</t>
         </is>
       </c>
+      <c r="O160" t="inlineStr">
+        <is>
+          <t>원인: * 복제가 프로젝트 전체 max(no)+1 을 주던 동안 시트 안 번호에 구멍이 쌓였다([SYM-42](https://linear.app/sym804/issue/SYM-42/bug-095-tc-복제가-프로젝트-전체-maxno1-을-줘서-시트-안-번호에-구멍이-난다)). 그 상태를 되돌리는 장치가 없었다
+수정 내용: * alembic f2b7c04e91a8 이 (project_id, sheet_name) 마다 no 를 1..N 으로 다시 매긴다. 순서는 바꾸지 않고 번호만 촏촏해진다
+* 지운 TC 는 살아 있는 번호 뒤로 민다. 그 자리에 두면 되살릴 때 겹친다
+* 순위를 CTE 가 아니라 임시 테이블에 담는다. 갱신 대상과 같은 테이블을 읽는 CTE 는 SQLite 가 인라인으로 펼치면 이미 바꾼 값 위에서 순위를 매긴다
+* 바꾸기 전 번호를 `_tc_no_backup_f2b7c04e91a8` 테이블에 남긴다. 되돌릴 수 없는 변경이라 대조할 것을 두었다</t>
+        </is>
+      </c>
+      <c r="P160" t="inlineStr">
+        <is>
+          <t>* 번호를 넣는 네 경로를 상위 이슈에서 모두 막았다([SYM-50](https://linear.app/sym804/issue/SYM-50/bug-102-tc-번호를-넣는-경로가-시트-안-순번-규약을-지키지-않는다)). 마이그레이션 하나로는 다음 임포트 한 번에 되돌아간다
+* `test_tc_no_normalize.py` 7건. 500행 시트로 실행 계획이 달라지는 구간까지 본다</t>
+        </is>
+      </c>
+      <c r="Q160" t="inlineStr">
+        <is>
+          <t>* 실 DB 23개 시트 중 규약을 어기던 13개가 정리됐다. TC 총계 2172건 그대로고 순서도 유지된다
+* TC 관리 화면의 No 와 TC 목록 엑셀이 달라진다. 수행 화면과 두 엑셀은 목록 순번이라 영향이 없다</t>
+        </is>
+      </c>
       <c r="R160" t="inlineStr">
         <is>
           <t>BE 1.4.1.0</t>
         </is>
       </c>
+      <c r="S160" t="inlineStr">
+        <is>
+          <t>* DB 0.8.1.0</t>
+        </is>
+      </c>
       <c r="T160" t="inlineStr">
         <is>
-          <t>미해결</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="U160" t="inlineStr">
@@ -12472,14 +12521,37 @@
           <t>- 코드 리뷰</t>
         </is>
       </c>
+      <c r="O161" t="inlineStr">
+        <is>
+          <t>원인: * 파이썬에서 max(no) 를 읽고 +1 해서 넣었다. 읽기와 쓰기 사이가 열려 있었고 제약도 없어 DB 가 막아 주지 않았다
+수정 내용: * `_next_no_expr()` 로 바꿨다. INSERT 문 안의 scalar subquery 로 세므로 그 창이 없다. SQL 로그로 INSERT 안에 SELECT 가 들어가는 것을 확인했다
+* 보장은 제약이 한다. `(project_id, sheet_name, no)` 부분 유니크 인덱스를 걸었다(a3d61f0c8be2)</t>
+        </is>
+      </c>
+      <c r="P161" t="inlineStr">
+        <is>
+          <t>* `test_tc_clone_concurrent.py` 2건(8병렬 복제). 다만 이 테스트는 **수정 전에도 통과했다**. SQLite 가 쓰기를 직렬화해서 실측 재현이 안 됐다
+* 즉 이 결함은 코드 경로로만 성립하고 실측으로는 못 봤다. 그래도 서브쿼리 방식은 비용이 없고 SQLite 의 직렬화에 기대지 않는 모양이라 그대로 둔다</t>
+        </is>
+      </c>
+      <c r="Q161" t="inlineStr">
+        <is>
+          <t>* TC 복제 두 경로(단건, 일괄)</t>
+        </is>
+      </c>
       <c r="R161" t="inlineStr">
         <is>
           <t>BE 1.4.1.0</t>
         </is>
       </c>
+      <c r="S161" t="inlineStr">
+        <is>
+          <t>* BE 1.4.2.0 / DB 0.8.1.0</t>
+        </is>
+      </c>
       <c r="T161" t="inlineStr">
         <is>
-          <t>미해결</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="U161" t="inlineStr">
@@ -12555,19 +12627,267 @@
           <t>- 코드 리뷰</t>
         </is>
       </c>
+      <c r="O162" t="inlineStr">
+        <is>
+          <t>원인: * 새니타이즈 함수가 TC 목록 내보내기 파일 안에만 있었다. 내보내기 경로가 셋인데 한 곳에만 두면 나머지는 뜼린 채로 남는다
+수정 내용: * `services/excel_safe.py` 로 빼서 세 경로가 같은 함수를 쓴다
+* 막는 시작 문자에 줄바꿈(\n)을 더했다. OWASP 목록에는 없지만 같은 계열이고 막아서 잃을 것이 없다</t>
+        </is>
+      </c>
+      <c r="P162" t="inlineStr">
+        <is>
+          <t>* `test_export_formula_injection.py` 4건. 세 내보내기를 모두 보고, 막아야 하는 시작 문자를 하나도 빠뜨렸는지 함수 단위로도 본다
+* 이 테스트는 원래 CI 에서 건너뛰어지고 있었다. 가드를 고쳐 지금은 기본 조건에서 돌다([SYM-49](https://linear.app/sym804/issue/SYM-49/bug-101-테스트-40건이-ci-에서-건너뛰어지고-있었다))</t>
+        </is>
+      </c>
+      <c r="Q162" t="inlineStr">
+        <is>
+          <t>* 수행 엑셀, 리포트 엑셀. TC 목록 내보내기는 원래 막혀 있었다</t>
+        </is>
+      </c>
       <c r="R162" t="inlineStr">
         <is>
           <t>BE 1.4.1.0</t>
         </is>
       </c>
+      <c r="S162" t="inlineStr">
+        <is>
+          <t>* BE 1.4.2.0</t>
+        </is>
+      </c>
       <c r="T162" t="inlineStr">
         <is>
-          <t>미해결</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="U162" t="inlineStr">
         <is>
           <t>SYM-48</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>BUG-101</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>bug</t>
+        </is>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>major</t>
+        </is>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>etc</t>
+        </is>
+      </c>
+      <c r="F163" t="inlineStr">
+        <is>
+          <t>테스트 40건이 CI 에서 건너뛰어지고 있었다</t>
+        </is>
+      </c>
+      <c r="G163" t="inlineStr">
+        <is>
+          <t>- 일부 테스트 파일이 CI 와 로컬 기본 실행에서 한 줄도 돌지 않는다
+- 그 안에 보안 수정(엑셀 수식 인젝션) 검증이 들어 있었다</t>
+        </is>
+      </c>
+      <c r="H163" t="inlineStr">
+        <is>
+          <t>- 개발 서버가 떠 있지 않으면 격리 환경이므로 전부 실행돼야 한다</t>
+        </is>
+      </c>
+      <c r="I163" t="inlineStr">
+        <is>
+          <t>- 기본 수집 262건, TEST_PORT 를 지정하면 302건. 40건 차이</t>
+        </is>
+      </c>
+      <c r="K163" t="inlineStr">
+        <is>
+          <t>1. 개발 서버를 내린다
+2. cd backend &amp;&amp; python -m pytest --collect-only -q
+3. 수집 건수를 TEST_PORT=8009 로 돌린 것과 비교한다</t>
+        </is>
+      </c>
+      <c r="L163" t="inlineStr">
+        <is>
+          <t>- 항상</t>
+        </is>
+      </c>
+      <c r="M163" t="inlineStr">
+        <is>
+          <t>- 수집 건수 262 대 302
+- .github/workflows/ci.yml 이 TEST_PORT 도 ALLOW_DEV_DB 도 주지 않는다</t>
+        </is>
+      </c>
+      <c r="N163" t="inlineStr">
+        <is>
+          <t>- 코드 리뷰</t>
+        </is>
+      </c>
+      <c r="O163" t="inlineStr">
+        <is>
+          <t>원인: - skip 가드가 포트 번호(:8008)로 판정했다
+- 그런데 conftest 는 개발 서버가 없으면 임시 DB 를 잡고 8008 에 격리 서버를 직접 띄운다. 그 상황은 위험하지 않은데도 건너뛰었다
+수정 내용: - backend/dev_db_guard.py 를 두고 conftest 가 실제 격리 여부를 채운다
+- 8개 파일이 포트가 아니라 그 값으로 판정한다
+- from conftest import 는 tests_unit/conftest.py 가 이름을 선점해 ImportError 가 나므로 별도 모듈로 뺐다</t>
+        </is>
+      </c>
+      <c r="P163" t="inlineStr">
+        <is>
+          <t>- 기본 조건에서 323건이 수집되고 전부 통과하는 것을 확인했다. 다음에 같은 가드를 복사해도 포트가 아니라 격리 여부를 본다</t>
+        </is>
+      </c>
+      <c r="Q163" t="inlineStr">
+        <is>
+          <t>- 백엔드 테스트 스위트 전체</t>
+        </is>
+      </c>
+      <c r="R163" t="inlineStr">
+        <is>
+          <t>BE 1.4.1.0</t>
+        </is>
+      </c>
+      <c r="S163" t="inlineStr">
+        <is>
+          <t>BE 1.4.2.0</t>
+        </is>
+      </c>
+      <c r="T163" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="U163" t="inlineStr">
+        <is>
+          <t>SYM-49</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>BUG-102</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>bug</t>
+        </is>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>major</t>
+        </is>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>db</t>
+        </is>
+      </c>
+      <c r="F164" t="inlineStr">
+        <is>
+          <t>TC 번호를 넣는 경로가 시트 안 순번 규약을 지키지 않는다</t>
+        </is>
+      </c>
+      <c r="G164" t="inlineStr">
+        <is>
+          <t>- 마이그레이션으로 번호를 1..N 으로 정리해도 다음 임포트나 드래그 한 번에 되돌아간다
+- 신규 생성, 임포트, 수정, 드래그 정렬이 각자 임의의 번호를 저장한다</t>
+        </is>
+      </c>
+      <c r="H164" t="inlineStr">
+        <is>
+          <t>- 살아 있는 TC 의 no 는 시트 안에서 1 부터 이어지고 겹치지 않는다</t>
+        </is>
+      </c>
+      <c r="I164" t="inlineStr">
+        <is>
+          <t>- 신규 생성이 클라이언트가 보낸 번호를 그대로 저장한다
+- 엑셀/CSV/마크다운 임포트가 파일의 No 를 그대로 저장한다
+- 드래그 정렬이 화면에 보이는 행만 1..N 으로 매겨 저장한다. 전체 보기면 시트 경계를 넘고, 검색 중이면 숨은 행이 빠진다
+- 수정 API 로 번호를 임의 값으로 바꿀 수 있다</t>
+        </is>
+      </c>
+      <c r="K164" t="inlineStr">
+        <is>
+          <t>1. 시트에 TC 를 세 건 만든다
+2. No 가 10, 20, 30 인 엑셀을 그 시트로 임포트한다
+3. TC 관리에서 그 시트의 No 를 본다</t>
+        </is>
+      </c>
+      <c r="L164" t="inlineStr">
+        <is>
+          <t>- 항상</t>
+        </is>
+      </c>
+      <c r="M164" t="inlineStr">
+        <is>
+          <t>- 새 테스트 test_tc_no_contract.py 15건이 수정 전에 절반 이상 실패했다</t>
+        </is>
+      </c>
+      <c r="N164" t="inlineStr">
+        <is>
+          <t>- 코드 리뷰</t>
+        </is>
+      </c>
+      <c r="O164" t="inlineStr">
+        <is>
+          <t>원인: - 번호를 서버가 관리하지 않고 클라이언트와 파일에 맡겼다. 제약도 없어 DB 가 막아 주지 않았다
+수정 내용: - 신규 생성이 클라이언트의 no 를 무시하고 INSERT 문 안에서 채번한다
+- 세 임포트 경로가 끝난 뒤 시트를 1..N 으로 맞춘다(services/tc_numbering.py)
+- 드래그 정렬은 한 시트 전체를 1..N 으로 보낼 때만 받는다. 아니면 400. 갱신은 음수로 밀었다가 목표값을 쓰는 2단계다
+- 수정 API 가 번호를 받지 않는다. 시트를 옮기면 양쪽 시트를 다시 매긴다
+- (project_id, sheet_name, no) 부분 유니크 인덱스로 DB 가 강제한다
+- 화면도 시트 탭이 활성이고 검색 중이 아닐 때만 드래그를 켜고, No 는 읽기 전용이다</t>
+        </is>
+      </c>
+      <c r="P164" t="inlineStr">
+        <is>
+          <t>- test_tc_no_contract.py 15건이 네 경로를 모두 본다
+- 인덱스가 있으므로 코드가 새도 DB 가 거절한다</t>
+        </is>
+      </c>
+      <c r="Q164" t="inlineStr">
+        <is>
+          <t>- TC 관리 화면의 No, TC 목록 엑셀, 임포트 결과</t>
+        </is>
+      </c>
+      <c r="R164" t="inlineStr">
+        <is>
+          <t>BE 1.4.1.0</t>
+        </is>
+      </c>
+      <c r="S164" t="inlineStr">
+        <is>
+          <t>BE 1.4.2.0 / FE 1.4.2.0 / DB 0.8.1.0</t>
+        </is>
+      </c>
+      <c r="T164" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="U164" t="inlineStr">
+        <is>
+          <t>SYM-50</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(import): 파일 번호에 걸려 임포트가 실패하던 문제 (v1.5.1.0, SYM-52/53)
앞 커밋이 시트 안 번호 규약을 DB 제약으로 세웠는데, 파일에서 번호를 읽는 세
경로 중 엑셀만 고쳐져 있었다.

- CSV 와 마크다운도 파일의 No 를 차례로만 쓴다. 파일 안에 같은 번호가 있으면
  409 로 통째로 죽었다. 사람이 만든 파일에서 흔한 경우다
- 번호를 비켜 두는 자리를 그 시트의 최대 절댓값보다 크게 잡는다. 고정 상수로
  두면 데이터에 그 값이 들어왔을 때 부딪친다. no = 0 인 행이 비켜지지 않던
  것도 같은 자리다
- 개발 DB 위험 판정이 테스트가 실제로 요청을 보내는 곳을 본다. TEST_PORT 만
  주면 판정은 빈 포트를 보고 안전하다 하는데 요청은 8008 로 갔다. 두 값이
  갈라지면 잡히는 테스트를 붙였고, 그 테스트가 가드 없는 파일 2개를 찾아냈다
- 정렬이 걸린 상태의 드래그를 저장 직전에 거절한다. 행 수가 같아 개수 비교로는
  걸리지 않는다. 판정을 화면 값 쓰기보다 앞으로 옮겨 거절 경로가 재조회 성공에
  의존하지 않게 했다
- 테스트 12건 추가. 백엔드 345건, 프론트 449건 통과

남긴 것: TC ID 가 없는 파일의 재임포트 매칭(SYM-51). 자동 생성 규칙을 바꾸면
이미 임포트된 프로젝트가 전부 새 행으로 잡혀 별도로 다룬다.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016UKFCyy7maLAXe6Si7ZiqR
</commit_message>
<xml_diff>
--- a/Issue_list.xlsx
+++ b/Issue_list.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U164"/>
+  <dimension ref="A1:U167"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -12891,6 +12891,305 @@
         </is>
       </c>
     </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>BUG-103</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>bug</t>
+        </is>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>minor</t>
+        </is>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>backend</t>
+        </is>
+      </c>
+      <c r="F165" t="inlineStr">
+        <is>
+          <t>TC ID 가 없는 파일을 다시 임포트하면 같은 행을 두 번 갱신할 수 있다</t>
+        </is>
+      </c>
+      <c r="G165" t="inlineStr">
+        <is>
+          <t>- TC ID 칸이 빈 파일을 두 번 임포트하면 일부 행이 갱신되지 않고 다른 행이 두 번 갱신된다</t>
+        </is>
+      </c>
+      <c r="H165" t="inlineStr">
+        <is>
+          <t>- 같은 파일을 다시 넣으면 같은 행이 한 번씩 갱신돼야 한다</t>
+        </is>
+      </c>
+      <c r="I165" t="inlineStr">
+        <is>
+          <t>- 파일에 같은 No 가 두 번 있으면 두 행 모두 같은 TC ID 로 계산된다. 첫 임포트에서는 TC-001 과 TC-001-2 로 갈라지지만, 두 번째 임포트에서는 둘 다 TC-001 을 찾는다</t>
+        </is>
+      </c>
+      <c r="K165" t="inlineStr">
+        <is>
+          <t>1. TC ID 칸이 비어 있고 No 가 1, 1 인 엑셀을 만든다
+2. 빈 시트에 임포트한다
+3. 같은 파일을 한 번 더 임포트한다
+4. 시트의 TC 를 본다</t>
+        </is>
+      </c>
+      <c r="L165" t="inlineStr">
+        <is>
+          <t>- 항상</t>
+        </is>
+      </c>
+      <c r="M165" t="inlineStr">
+        <is>
+          <t>- import_service.py 의 세 파서가 TC ID 가 없으면 파일의 No 로 TC-{no:03d} 를 만든다. 저장하는 no 는 행 순번으로 바꿨지만 이 생성 규칙은 그대로다</t>
+        </is>
+      </c>
+      <c r="N165" t="inlineStr">
+        <is>
+          <t>- 코드 리뷰</t>
+        </is>
+      </c>
+      <c r="R165" t="inlineStr">
+        <is>
+          <t>BE 1.5.0.0</t>
+        </is>
+      </c>
+      <c r="T165" t="inlineStr">
+        <is>
+          <t>미해결</t>
+        </is>
+      </c>
+      <c r="U165" t="inlineStr">
+        <is>
+          <t>SYM-51</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>BUG-104</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>bug</t>
+        </is>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>major</t>
+        </is>
+      </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>backend</t>
+        </is>
+      </c>
+      <c r="F166" t="inlineStr">
+        <is>
+          <t>파일 안에 같은 번호가 있으면 CSV 와 마크다운 임포트가 통째로 실패한다</t>
+        </is>
+      </c>
+      <c r="G166" t="inlineStr">
+        <is>
+          <t>- No 가 겹치는 CSV 나 마크다운을 임포트하면 409 '데이터 제약 조건에 걸렸습니다' 로 아무것도 들어가지 않는다</t>
+        </is>
+      </c>
+      <c r="H166" t="inlineStr">
+        <is>
+          <t>- 파일의 번호와 무관하게 받아들이고 시트 안에서 1..N 으로 정리돼야 한다</t>
+        </is>
+      </c>
+      <c r="I166" t="inlineStr">
+        <is>
+          <t>- 파서가 파일의 No 를 그대로 저장해 유니크 제약에 걸린다. 엑셀만 행 순서로 붙이도록 고쳐져 있었다</t>
+        </is>
+      </c>
+      <c r="K166" t="inlineStr">
+        <is>
+          <t>1. No 가 1, 1 인 두 줄짜리 CSV 를 만든다
+2. 아무 프로젝트에 임포트한다</t>
+        </is>
+      </c>
+      <c r="L166" t="inlineStr">
+        <is>
+          <t>- 항상</t>
+        </is>
+      </c>
+      <c r="M166" t="inlineStr">
+        <is>
+          <t>- 재현 테스트가 409 를 받았다. 파서 수정을 되돌리면 다시 실패한다</t>
+        </is>
+      </c>
+      <c r="N166" t="inlineStr">
+        <is>
+          <t>- 코드 리뷰</t>
+        </is>
+      </c>
+      <c r="O166" t="inlineStr">
+        <is>
+          <t>원인: - 앞 릴리즈에서 시트 안 번호 규약을 세우며 엑셀 파서만 고쳤다. CSV 와 마크다운은 파일의 No 를 int 로 바꿔 그대로 넣는다
+- 유니크 인덱스를 걸기 전에는 중복이 저장됐다가 뒤에서 정리됐는데, 인덱스를 건 뒤로는 정리 코드에 닿지 못한다
+수정 내용: - 두 파서가 파일의 No 를 차례로만 쓰고 행 순번을 저장한다
+- 임포트 앞에서 그 시트의 번호를 비켜 두는 자리를 고정 상수가 아니라 시트의 최대 절댓값보다 크게 잡는다. 상수로 두면 데이터에 그 값이 들어왔을 때 부딪친다</t>
+        </is>
+      </c>
+      <c r="P166" t="inlineStr">
+        <is>
+          <t>- 파일 안 중복 번호, 음수 번호, 같은 시트 두 번 임포트를 보는 테스트를 세 파일 형식마다 뒀다
+- 재번호 함수를 유니크 인덱스가 걸린 테이블에서 직접 부르는 단위 테스트 11건</t>
+        </is>
+      </c>
+      <c r="Q166" t="inlineStr">
+        <is>
+          <t>- CSV, 마크다운 임포트</t>
+        </is>
+      </c>
+      <c r="R166" t="inlineStr">
+        <is>
+          <t>BE 1.5.0.0</t>
+        </is>
+      </c>
+      <c r="S166" t="inlineStr">
+        <is>
+          <t>BE 1.5.1.0</t>
+        </is>
+      </c>
+      <c r="T166" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="U166" t="inlineStr">
+        <is>
+          <t>SYM-52</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>BUG-105</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>bug</t>
+        </is>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>major</t>
+        </is>
+      </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>etc</t>
+        </is>
+      </c>
+      <c r="F167" t="inlineStr">
+        <is>
+          <t>개발 DB 를 지키는 테스트 가드가 실제 요청 대상을 보지 않는다</t>
+        </is>
+      </c>
+      <c r="G167" t="inlineStr">
+        <is>
+          <t>- 격리됐다고 판정하면서 요청은 개발 서버로 가는 조합이 있다</t>
+        </is>
+      </c>
+      <c r="H167" t="inlineStr">
+        <is>
+          <t>- 테스트가 실제로 요청을 보내는 곳에 개발 서버가 떠 있으면 건너뛰어야 한다</t>
+        </is>
+      </c>
+      <c r="I167" t="inlineStr">
+        <is>
+          <t>- 판정은 TEST_PORT 를 보는데 테스트 모듈은 TEST_BASE_URL 이 없으면 8008 로 간다. TEST_PORT=8009 만 주면 판정은 안전하다 하고 요청은 개발 서버로 간다
+- 가드가 아예 없는 HTTP 테스트도 2개 있었다</t>
+        </is>
+      </c>
+      <c r="K167" t="inlineStr">
+        <is>
+          <t>1. 개발 서버를 8008 에 띄운다
+2. TEST_PORT=8009 만 주고 pytest 를 돌린다
+3. 요청이 어디로 가는지 본다</t>
+        </is>
+      </c>
+      <c r="L167" t="inlineStr">
+        <is>
+          <t>- 항상</t>
+        </is>
+      </c>
+      <c r="M167" t="inlineStr">
+        <is>
+          <t>- 테스트 모듈의 기본 주소가 리터럴 8008 이고 conftest 의 폴백은 TEST_PORT 였다</t>
+        </is>
+      </c>
+      <c r="N167" t="inlineStr">
+        <is>
+          <t>- 코드 리뷰</t>
+        </is>
+      </c>
+      <c r="O167" t="inlineStr">
+        <is>
+          <t>원인: - 판정 기준과 요청 대상이 각자 기본값을 들고 있어 조용히 갈라졌다
+수정 내용: - 기본 포트를 dev_db_guard 한 곳에 두고 conftest 가 그것을 참조한다
+- 두 값이 갈라지면 실패하는 테스트를 붙였다. 그 테스트가 가드 없는 파일 2개를 찾아냈고 거기에도 가드를 달았다</t>
+        </is>
+      </c>
+      <c r="P167" t="inlineStr">
+        <is>
+          <t>- test_dev_db_guard.py 가 기본 포트 일치, 가드 존재, conftest 의 폴백 참조를 대조한다. conftest 를 리터럴로 되돌리면 실패한다</t>
+        </is>
+      </c>
+      <c r="Q167" t="inlineStr">
+        <is>
+          <t>- 백엔드 테스트 스위트</t>
+        </is>
+      </c>
+      <c r="R167" t="inlineStr">
+        <is>
+          <t>BE 1.5.0.0</t>
+        </is>
+      </c>
+      <c r="S167" t="inlineStr">
+        <is>
+          <t>BE 1.5.1.0</t>
+        </is>
+      </c>
+      <c r="T167" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="U167" t="inlineStr">
+        <is>
+          <t>SYM-53</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix(export): TC 0건 프로젝트의 시트 분리 내보내기 실패 (v1.5.3.0, SYM-60/61)
시트 분리 모드는 기본 시트를 지운 뒤 TC 의 sheet_name 별로 탭을 만든다.
TC 가 0건이면 탭이 하나도 남지 않아 openpyxl 이 저장 단계에서
IndexError("At least one sheet must be visible") 를 던지고 500 이 된다.
전체 TC 가 소프트 삭제된 프로젝트도 같은 경로를 탄다.

- sheets_map 이 비면 Test Cases 한 장을 넣어 통합 모드와 결과를 맞춘다
- 시트명 정제를 _safe_sheet_title 로 모으고 31자 상한 안에서 중복을 푼다.
  종전에는 정제 전에 자르느라 앞 31자가 같은 이름이 충돌했고, openpyxl 이
  붙인 번호가 상한 밖으로 나가 32자 탭이 생겼다(실측 [5, 3, 4, 31, 32])
- 금지 문자만 남아 이름이 비면 기본 으로 채운다
- 회귀 체크리스트에 TC-EXP-001/002/003 추가

QA 2인 통과. 두 QA 모두 "금지 문자만 있는 이름은 ValueError 로 500" 이라고
봤으나 실측에서는 openpyxl 이 Sheet 로 대체해 저장된다. 대신 31자 초과가
실제 결함이었다. 신규 테스트 5건, 고의 결함 주입으로 검출 확인.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AuvUeSrxUUKqFVwzsfoqwu
</commit_message>
<xml_diff>
--- a/Issue_list.xlsx
+++ b/Issue_list.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U173"/>
+  <dimension ref="A1:U175"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -13784,6 +13784,214 @@
         </is>
       </c>
     </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>BUG-111</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>bug</t>
+        </is>
+      </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>major</t>
+        </is>
+      </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>backend</t>
+        </is>
+      </c>
+      <c r="F174" t="inlineStr">
+        <is>
+          <t>TC 가 없는 프로젝트에서 시트 분리 내보내기가 500 으로 실패한다</t>
+        </is>
+      </c>
+      <c r="G174" t="inlineStr">
+        <is>
+          <t>- TC 관리 탭의 Excel Export 에서 시트 분리를 고르면 오류 토스트만 뜨고 파일이 내려오지 않는다.
+- 시트 통합으로 고르면 정상으로 내려온다.</t>
+        </is>
+      </c>
+      <c r="H174" t="inlineStr">
+        <is>
+          <t>- 두 모드 모두 파일이 내려온다. TC 가 없으면 헤더만 있는 파일이 나온다.</t>
+        </is>
+      </c>
+      <c r="I174" t="inlineStr">
+        <is>
+          <t>- GET /api/projects/19/testcases/export?split_sheets=true 가 500 과 Internal server error 를 낸다.</t>
+        </is>
+      </c>
+      <c r="K174" t="inlineStr">
+        <is>
+          <t>1. TC 가 한 건도 없는 프로젝트를 연다.
+2. TC 관리 탭에서 Excel Export 를 누른다.
+3. 시트 분리 (시트별 탭) 를 고르고 다운로드를 누른다.</t>
+        </is>
+      </c>
+      <c r="L174" t="inlineStr">
+        <is>
+          <t>- 항상</t>
+        </is>
+      </c>
+      <c r="M174" t="inlineStr">
+        <is>
+          <t>- IndexError: At least one sheet must be visible (openpyxl/workbook/_writer.py:35)
+- 같은 프로젝트에서 split_sheets=false 는 200 / 5454 bytes.</t>
+        </is>
+      </c>
+      <c r="N174" t="inlineStr">
+        <is>
+          <t>- 사용자</t>
+        </is>
+      </c>
+      <c r="O174" t="inlineStr">
+        <is>
+          <t>원인: - export_service 가 wb.remove(wb.active) 로 기본 시트를 지운 뒤 TC 의 sheet_name 별로 탭을 만든다.
+- TC 가 0건이면 sheets_map 이 비어 탭이 하나도 생기지 않고, 시트 0개인 워크북은 저장 단계에서 죽는다.
+- 전체 TC 가 소프트 삭제된 프로젝트도 조회 결과가 빈 목록이라 같은 경로를 탄다.
+수정 내용: - sheets_map 이 비면 Test Cases 한 장을 넣어 통합 모드와 같은 결과를 낸다.
+- 시트명 정제를 _safe_sheet_title 헬퍼로 모으고 31자 상한과 중복 회피를 함께 처리한다.</t>
+        </is>
+      </c>
+      <c r="P174" t="inlineStr">
+        <is>
+          <t>- backend/test_export_empty_project.py 5건 추가. 고의 결함 주입으로 검출 여부를 확인했다.
+- 회귀 체크리스트에 TC-EXP-001/002/003 추가.</t>
+        </is>
+      </c>
+      <c r="Q174" t="inlineStr">
+        <is>
+          <t>- TC 목록 엑셀 내보내기의 시트 분리 모드. 런 엑셀과 리포트 엑셀은 시트를 항상 만들어 해당 없음.</t>
+        </is>
+      </c>
+      <c r="R174" t="inlineStr">
+        <is>
+          <t>BE 1.5.2.0</t>
+        </is>
+      </c>
+      <c r="T174" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="U174" t="inlineStr">
+        <is>
+          <t>SYM-60</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>BUG-112</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>bug</t>
+        </is>
+      </c>
+      <c r="D175" t="inlineStr">
+        <is>
+          <t>minor</t>
+        </is>
+      </c>
+      <c r="E175" t="inlineStr">
+        <is>
+          <t>backend</t>
+        </is>
+      </c>
+      <c r="F175" t="inlineStr">
+        <is>
+          <t>시트명이 31자를 넘고 서로 겹치면 엑셀 탭 이름이 32자가 된다</t>
+        </is>
+      </c>
+      <c r="G175" t="inlineStr">
+        <is>
+          <t>- 시트 분리로 내보낸 파일의 탭 이름이 엑셀 상한인 31자를 넘는다.</t>
+        </is>
+      </c>
+      <c r="H175" t="inlineStr">
+        <is>
+          <t>- 모든 탭 이름이 31자 이하이고 서로 겹치지 않는다.</t>
+        </is>
+      </c>
+      <c r="I175" t="inlineStr">
+        <is>
+          <t>- 앞 31자가 같은 시트 두 개를 만들어 내보내니 탭 이름이 32자로 나왔다.</t>
+        </is>
+      </c>
+      <c r="K175" t="inlineStr">
+        <is>
+          <t>1. 앞 31자가 같고 뒤만 다른 시트 두 개를 만든다.
+2. 각 시트에 TC 를 한 건씩 넣는다.
+3. 시트 분리로 내보내고 탭 이름 길이를 확인한다.</t>
+        </is>
+      </c>
+      <c r="L175" t="inlineStr">
+        <is>
+          <t>- 항상</t>
+        </is>
+      </c>
+      <c r="M175" t="inlineStr">
+        <is>
+          <t>- 탭 이름 길이 실측: [5, 3, 4, 31, 32]. 마지막 항목이 상한을 넘는다.</t>
+        </is>
+      </c>
+      <c r="N175" t="inlineStr">
+        <is>
+          <t>- 코드 리뷰</t>
+        </is>
+      </c>
+      <c r="O175" t="inlineStr">
+        <is>
+          <t>원인: - 정제 전에 31자로 자르기 때문에 앞부분이 같은 이름끼리 충돌한다.
+- openpyxl 은 중복 제목을 만나면 뒤에 번호를 붙이는데 그 번호가 상한 밖으로 나간다.
+수정 내용: - _safe_sheet_title 이 정제와 자르기를 한 자리에서 하고, 충돌하면 번호까지 포함해 31자 안에 넣는다.
+- 금지 문자만 남아 이름이 비면 기본 으로 채운다.</t>
+        </is>
+      </c>
+      <c r="P175" t="inlineStr">
+        <is>
+          <t>- test_export_empty_project.py 에 31자 상한과 금지 문자 케이스 테스트 추가.</t>
+        </is>
+      </c>
+      <c r="Q175" t="inlineStr">
+        <is>
+          <t>- TC 목록 엑셀 내보내기의 시트 분리 모드. 기존 프로젝트 9개 탭 이름은 수정 전후 동일하다.</t>
+        </is>
+      </c>
+      <c r="R175" t="inlineStr">
+        <is>
+          <t>BE 1.5.2.0</t>
+        </is>
+      </c>
+      <c r="T175" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="U175" t="inlineStr">
+        <is>
+          <t>SYM-61</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(dev): 로컬 구동과 API 호출을 devctl 한 자리로 (SYM-62)
서버를 띄우고 인증 API 를 부르는 일을 매번 손으로 조립했다. 한 세션에서
여섯 번 넘게 반복했고 그 사이 두 번 틀렸다. 옛 uvicorn 이 포트를 쥔 채
수정 전 코드로 응답했고, netstat -p TCP 가 IPv4 만 내는 줄 모르고 프론트
서버를 내려간 것으로 읽었다.

- scripts/devctl.py: up / down / status / token / api
  - up 은 기존 리스너를 먼저 정리한다
  - PID 는 포트 기준으로만 찾는다. 이름으로 죽이지 않는다
  - 비밀번호는 TCM_ADMIN_PW 또는 account.txt(gitignore)에서 읽는다
  - Git Bash 의 /api 경로 변환과 vite 의 IPv6 바인딩을 도구가 흡수한다
- .claude/skills/dev: 포트, DB 위치, 브라우저 확인 절차, 함정
- .gitignore: 개인 설정은 빼고 프로젝트 스킬만 추적. 루트 skills/ 규칙에
  앞 슬래시가 없어 .claude/skills/ 까지 걸리던 것도 함께 고침

제품 런타임 코드는 바뀌지 않아 버전은 올리지 않는다.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AuvUeSrxUUKqFVwzsfoqwu
</commit_message>
<xml_diff>
--- a/Issue_list.xlsx
+++ b/Issue_list.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U175"/>
+  <dimension ref="A1:U176"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -13992,6 +13992,98 @@
         </is>
       </c>
     </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>ENH-048</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>enhancement</t>
+        </is>
+      </c>
+      <c r="D176" t="inlineStr">
+        <is>
+          <t>minor</t>
+        </is>
+      </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>etc</t>
+        </is>
+      </c>
+      <c r="F176" t="inlineStr">
+        <is>
+          <t>로컬 구동과 API 호출을 devctl 한 자리로 모은다</t>
+        </is>
+      </c>
+      <c r="G176" t="inlineStr">
+        <is>
+          <t>- 서버를 띄울 때마다 uvicorn 명령을 손으로 조립한다.
+- 인증이 필요한 API 를 부르려면 로그인, 토큰 추출, curl 조립을 매번 반복한다.
+- run_dev.sh 는 포그라운드로 잡고 Ctrl+C 를 기다려 자동화에서 쓸 수 없다.</t>
+        </is>
+      </c>
+      <c r="H176" t="inlineStr">
+        <is>
+          <t>- scripts/devctl.py 의 up, down, status, token, api 로 끝난다.
+- up 이 기존 프로세스를 먼저 정리하므로 옛 코드가 응답하는 사고가 나지 않는다.
+- .claude/skills/dev 에 포트, DB 위치, 브라우저 확인 절차, 함정을 적어 둔다.</t>
+        </is>
+      </c>
+      <c r="K176" t="inlineStr">
+        <is>
+          <t>- [x] up, down, status, token, api 가 모두 동작한다
+- [x] 포트를 LISTEN 하는 PID 만 종료한다
+- [x] 비밀번호가 코드에 없다
+- [x] 프로젝트 스킬이 레포에 추적된다</t>
+        </is>
+      </c>
+      <c r="N176" t="inlineStr">
+        <is>
+          <t>- 한 번의 작업에서 로그인과 토큰 조립을 여섯 번 넘게 반복했다.
+- 그 과정에서 실제로 두 번 틀렸다. 옛 uvicorn 이 살아 있어 수정 전 코드가 응답했고, 프론트 PID 를 못 찾아 서버가 내려간 줄 알고 방치했다.</t>
+        </is>
+      </c>
+      <c r="O176" t="inlineStr">
+        <is>
+          <t>- devctl.py 추가, .claude/skills/dev/SKILL.md 추가, .gitignore 에서 프로젝트 스킬만 추적하도록 예외 지정.
+- Git Bash 의 경로 변환과 vite 의 IPv6 바인딩을 도구가 흡수한다.</t>
+        </is>
+      </c>
+      <c r="P176" t="inlineStr">
+        <is>
+          <t>- 다른 프로젝트로 일반화. ym-testcase 에서 쓸모를 확인한 뒤에 판단한다.
+- run_dev.sh 대체. 사람이 터미널에서 쓰는 용도는 그대로 둔다.</t>
+        </is>
+      </c>
+      <c r="Q176" t="inlineStr">
+        <is>
+          <t>- 개발 편의 도구. 제품 런타임 코드는 바뀌지 않는다.</t>
+        </is>
+      </c>
+      <c r="R176" t="inlineStr">
+        <is>
+          <t>BE 1.5.3.0</t>
+        </is>
+      </c>
+      <c r="T176" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="U176" t="inlineStr">
+        <is>
+          <t>SYM-62</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>